<commit_message>
16 DECEMBER 2025 13.46
</commit_message>
<xml_diff>
--- a/DECEMBER/DECEMBER BAR.xlsx
+++ b/DECEMBER/DECEMBER BAR.xlsx
@@ -105,7 +105,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="400" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="422" uniqueCount="119">
   <si>
     <t>DATE</t>
   </si>
@@ -215,6 +215,15 @@
     <t>APPLE</t>
   </si>
   <si>
+    <t>GREEN APPLE</t>
+  </si>
+  <si>
+    <t>SARIWANGI TEA</t>
+  </si>
+  <si>
+    <t>BEETROOT</t>
+  </si>
+  <si>
     <t>INV NO</t>
   </si>
   <si>
@@ -288,9 +297,6 @@
   </si>
   <si>
     <t>PINEAPPLE</t>
-  </si>
-  <si>
-    <t>GREEN APPLE</t>
   </si>
   <si>
     <t>STRAWBERRY</t>
@@ -1478,7 +1484,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="301">
+  <cellXfs count="309">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -2371,6 +2377,30 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="181" fontId="30" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="181" fontId="30" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="181" fontId="30" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="180" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3496,7 +3526,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:H391"/>
+  <dimension ref="A1:H400"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="16.8" outlineLevelCol="7"/>
   <cols>
     <col min="1" max="1" width="17.5703125" style="251" customWidth="1"/>
@@ -4940,7 +4970,7 @@
         <v>48000</v>
       </c>
       <c r="E82" s="7">
-        <f t="shared" ref="E82:E145" si="5">SUM(C82*D82)</f>
+        <f>SUM(C82*D82)</f>
         <v>96000</v>
       </c>
       <c r="F82" s="294"/>
@@ -4973,7 +5003,7 @@
         <v>20000</v>
       </c>
       <c r="E84" s="7">
-        <f t="shared" si="5"/>
+        <f>SUM(C84*D84)</f>
         <v>6000</v>
       </c>
       <c r="F84" s="294"/>
@@ -4990,7 +5020,7 @@
         <v>30000</v>
       </c>
       <c r="E85" s="7">
-        <f t="shared" si="5"/>
+        <f>SUM(C85*D85)</f>
         <v>15000</v>
       </c>
       <c r="F85" s="294"/>
@@ -5007,7 +5037,7 @@
         <v>80000</v>
       </c>
       <c r="E86" s="7">
-        <f t="shared" si="5"/>
+        <f>SUM(C86*D86)</f>
         <v>40000</v>
       </c>
       <c r="F86" s="294"/>
@@ -5041,7 +5071,7 @@
         <v>15000</v>
       </c>
       <c r="E88" s="7">
-        <f t="shared" si="5"/>
+        <f>SUM(C88*D88)</f>
         <v>15000</v>
       </c>
       <c r="F88" s="294"/>
@@ -5058,7 +5088,7 @@
         <v>24000</v>
       </c>
       <c r="E89" s="7">
-        <f t="shared" si="5"/>
+        <f>SUM(C89*D89)</f>
         <v>48000</v>
       </c>
       <c r="F89" s="294"/>
@@ -5075,7 +5105,7 @@
         <v>40000</v>
       </c>
       <c r="E90" s="7">
-        <f t="shared" si="5"/>
+        <f>SUM(C90*D90)</f>
         <v>40000</v>
       </c>
       <c r="F90" s="294"/>
@@ -5092,7 +5122,7 @@
         <v>49000</v>
       </c>
       <c r="E91" s="7">
-        <f t="shared" si="5"/>
+        <f>SUM(C91*D91)</f>
         <v>49000</v>
       </c>
       <c r="F91" s="294"/>
@@ -5109,7 +5139,7 @@
         <v>20000</v>
       </c>
       <c r="E92" s="7">
-        <f t="shared" si="5"/>
+        <f>SUM(C92*D92)</f>
         <v>80000</v>
       </c>
       <c r="F92" s="294"/>
@@ -5126,7 +5156,7 @@
         <v>20000</v>
       </c>
       <c r="E93" s="7">
-        <f t="shared" si="5"/>
+        <f>SUM(C93*D93)</f>
         <v>80000</v>
       </c>
       <c r="F93" s="295"/>
@@ -5145,7 +5175,7 @@
         <v>10000</v>
       </c>
       <c r="E94" s="7">
-        <f t="shared" si="5"/>
+        <f>SUM(C94*D94)</f>
         <v>80000</v>
       </c>
       <c r="F94" s="293">
@@ -5181,7 +5211,7 @@
         <v>38000</v>
       </c>
       <c r="E96" s="7">
-        <f t="shared" si="5"/>
+        <f>SUM(C96*D96)</f>
         <v>76000</v>
       </c>
       <c r="F96" s="294"/>
@@ -5198,7 +5228,7 @@
         <v>20000</v>
       </c>
       <c r="E97" s="7">
-        <f t="shared" si="5"/>
+        <f>SUM(C97*D97)</f>
         <v>40000</v>
       </c>
       <c r="F97" s="294"/>
@@ -5215,7 +5245,7 @@
         <v>24000</v>
       </c>
       <c r="E98" s="7">
-        <f t="shared" si="5"/>
+        <f>SUM(C98*D98)</f>
         <v>96000</v>
       </c>
       <c r="F98" s="294"/>
@@ -5232,258 +5262,391 @@
         <v>40000</v>
       </c>
       <c r="E99" s="7">
+        <f>SUM(C99*D99)</f>
+        <v>80000</v>
+      </c>
+      <c r="F99" s="295"/>
+    </row>
+    <row r="100" s="249" customFormat="1" ht="14" customHeight="1" spans="1:6">
+      <c r="A100" s="298">
+        <v>46005</v>
+      </c>
+      <c r="B100" s="290" t="s">
+        <v>8</v>
+      </c>
+      <c r="C100" s="297">
+        <v>8</v>
+      </c>
+      <c r="D100" s="7">
+        <v>10000</v>
+      </c>
+      <c r="E100" s="22">
+        <f t="shared" ref="E100:E108" si="5">SUM(C100*D100)</f>
+        <v>80000</v>
+      </c>
+      <c r="F100" s="301">
+        <f>SUM(E100:E108)</f>
+        <v>506000</v>
+      </c>
+    </row>
+    <row r="101" s="249" customFormat="1" ht="14" customHeight="1" spans="1:6">
+      <c r="A101" s="298"/>
+      <c r="B101" s="290" t="s">
+        <v>24</v>
+      </c>
+      <c r="C101" s="297">
+        <v>8.23</v>
+      </c>
+      <c r="D101" s="7">
+        <v>15000</v>
+      </c>
+      <c r="E101" s="22">
+        <v>123000</v>
+      </c>
+      <c r="F101" s="302"/>
+    </row>
+    <row r="102" s="249" customFormat="1" ht="14" customHeight="1" spans="1:6">
+      <c r="A102" s="298"/>
+      <c r="B102" s="290" t="s">
+        <v>6</v>
+      </c>
+      <c r="C102" s="297">
+        <v>2</v>
+      </c>
+      <c r="D102" s="7">
+        <v>20000</v>
+      </c>
+      <c r="E102" s="22">
         <f t="shared" si="5"/>
-        <v>80000</v>
-      </c>
-      <c r="F99" s="295"/>
-    </row>
-    <row r="100" s="249" customFormat="1" ht="14" customHeight="1" spans="1:6">
-      <c r="A100" s="291"/>
-      <c r="B100" s="290"/>
-      <c r="C100" s="297"/>
-      <c r="D100" s="7"/>
-      <c r="E100" s="7">
+        <v>40000</v>
+      </c>
+      <c r="F102" s="302"/>
+    </row>
+    <row r="103" s="249" customFormat="1" ht="14" customHeight="1" spans="1:6">
+      <c r="A103" s="298"/>
+      <c r="B103" s="290" t="s">
+        <v>10</v>
+      </c>
+      <c r="C103" s="297">
+        <v>0.3</v>
+      </c>
+      <c r="D103" s="7">
+        <v>20000</v>
+      </c>
+      <c r="E103" s="22">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="F100" s="298"/>
-    </row>
-    <row r="101" s="249" customFormat="1" ht="14" customHeight="1" spans="1:6">
-      <c r="A101" s="291"/>
-      <c r="B101" s="290"/>
-      <c r="C101" s="297"/>
-      <c r="D101" s="7"/>
-      <c r="E101" s="7">
+        <v>6000</v>
+      </c>
+      <c r="F103" s="302"/>
+    </row>
+    <row r="104" s="249" customFormat="1" ht="14" customHeight="1" spans="1:6">
+      <c r="A104" s="298"/>
+      <c r="B104" s="290" t="s">
+        <v>13</v>
+      </c>
+      <c r="C104" s="297">
+        <v>1</v>
+      </c>
+      <c r="D104" s="7">
+        <v>15000</v>
+      </c>
+      <c r="E104" s="22">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="F101" s="298"/>
-    </row>
-    <row r="102" s="249" customFormat="1" ht="14" customHeight="1" spans="1:6">
-      <c r="A102" s="291"/>
-      <c r="B102" s="290"/>
-      <c r="C102" s="297"/>
-      <c r="D102" s="7"/>
-      <c r="E102" s="7">
+        <v>15000</v>
+      </c>
+      <c r="F104" s="302"/>
+    </row>
+    <row r="105" s="249" customFormat="1" ht="14" customHeight="1" spans="1:6">
+      <c r="A105" s="298"/>
+      <c r="B105" s="290" t="s">
+        <v>36</v>
+      </c>
+      <c r="C105" s="297">
+        <v>1</v>
+      </c>
+      <c r="D105" s="7">
+        <v>48000</v>
+      </c>
+      <c r="E105" s="22">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="F102" s="298"/>
-    </row>
-    <row r="103" s="249" customFormat="1" ht="14" customHeight="1" spans="1:6">
-      <c r="A103" s="291"/>
-      <c r="B103" s="290"/>
-      <c r="C103" s="297"/>
-      <c r="D103" s="7"/>
-      <c r="E103" s="7">
+        <v>48000</v>
+      </c>
+      <c r="F105" s="302"/>
+    </row>
+    <row r="106" s="249" customFormat="1" ht="14" customHeight="1" spans="1:6">
+      <c r="A106" s="298"/>
+      <c r="B106" s="290" t="s">
+        <v>14</v>
+      </c>
+      <c r="C106" s="297">
+        <v>5</v>
+      </c>
+      <c r="D106" s="7">
+        <v>24000</v>
+      </c>
+      <c r="E106" s="22">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="F103" s="298"/>
-    </row>
-    <row r="104" s="249" customFormat="1" ht="14" customHeight="1" spans="1:6">
-      <c r="A104" s="291"/>
-      <c r="B104" s="290"/>
-      <c r="C104" s="297"/>
-      <c r="D104" s="7"/>
-      <c r="E104" s="7">
+        <v>120000</v>
+      </c>
+      <c r="F106" s="302"/>
+    </row>
+    <row r="107" s="249" customFormat="1" ht="14" customHeight="1" spans="1:6">
+      <c r="A107" s="298"/>
+      <c r="B107" s="290" t="s">
+        <v>32</v>
+      </c>
+      <c r="C107" s="297">
+        <v>1</v>
+      </c>
+      <c r="D107" s="7">
+        <v>49000</v>
+      </c>
+      <c r="E107" s="22">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="F104" s="298">
-        <f>SUM(E104:E118)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="105" s="249" customFormat="1" ht="14" customHeight="1" spans="1:6">
-      <c r="A105" s="291"/>
-      <c r="B105" s="290"/>
-      <c r="C105" s="297"/>
-      <c r="D105" s="7"/>
-      <c r="E105" s="7">
+        <v>49000</v>
+      </c>
+      <c r="F107" s="302"/>
+    </row>
+    <row r="108" s="249" customFormat="1" ht="14" customHeight="1" spans="1:6">
+      <c r="A108" s="298"/>
+      <c r="B108" s="290" t="s">
+        <v>37</v>
+      </c>
+      <c r="C108" s="297">
+        <v>1</v>
+      </c>
+      <c r="D108" s="7">
+        <v>25000</v>
+      </c>
+      <c r="E108" s="22">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="F105" s="298"/>
-    </row>
-    <row r="106" s="249" customFormat="1" ht="14" customHeight="1" spans="1:6">
-      <c r="A106" s="291"/>
-      <c r="B106" s="290"/>
-      <c r="C106" s="297"/>
-      <c r="D106" s="7"/>
-      <c r="E106" s="7">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="F106" s="298"/>
-    </row>
-    <row r="107" s="249" customFormat="1" ht="14" customHeight="1" spans="1:6">
-      <c r="A107" s="291"/>
-      <c r="B107" s="290"/>
-      <c r="C107" s="297"/>
-      <c r="D107" s="7"/>
-      <c r="E107" s="7">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="F107" s="298"/>
-    </row>
-    <row r="108" s="249" customFormat="1" ht="14" customHeight="1" spans="1:6">
-      <c r="A108" s="291"/>
-      <c r="B108" s="290"/>
-      <c r="C108" s="297"/>
-      <c r="D108" s="7"/>
-      <c r="E108" s="7">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="F108" s="298"/>
+        <v>25000</v>
+      </c>
+      <c r="F108" s="302"/>
     </row>
     <row r="109" s="249" customFormat="1" ht="14" customHeight="1" spans="1:6">
-      <c r="A109" s="291"/>
-      <c r="B109" s="290"/>
-      <c r="C109" s="297"/>
-      <c r="D109" s="7"/>
+      <c r="A109" s="299">
+        <v>46006</v>
+      </c>
+      <c r="B109" s="290" t="s">
+        <v>8</v>
+      </c>
+      <c r="C109" s="297">
+        <v>4</v>
+      </c>
+      <c r="D109" s="7">
+        <v>10000</v>
+      </c>
       <c r="E109" s="7">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="F109" s="298"/>
+        <f t="shared" ref="E109:E154" si="6">SUM(C109*D109)</f>
+        <v>40000</v>
+      </c>
+      <c r="F109" s="303">
+        <f>SUM(E109:E121)</f>
+        <v>630000</v>
+      </c>
     </row>
     <row r="110" s="249" customFormat="1" ht="14" customHeight="1" spans="1:6">
-      <c r="A110" s="291"/>
-      <c r="B110" s="290"/>
-      <c r="C110" s="297"/>
-      <c r="D110" s="7"/>
+      <c r="A110" s="298"/>
+      <c r="B110" s="290" t="s">
+        <v>24</v>
+      </c>
+      <c r="C110" s="297">
+        <v>3.43</v>
+      </c>
+      <c r="D110" s="7">
+        <v>15000</v>
+      </c>
       <c r="E110" s="7">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="F110" s="298"/>
+        <v>51000</v>
+      </c>
+      <c r="F110" s="304"/>
     </row>
     <row r="111" s="249" customFormat="1" ht="14" customHeight="1" spans="1:6">
-      <c r="A111" s="291"/>
-      <c r="B111" s="290"/>
-      <c r="C111" s="297"/>
-      <c r="D111" s="7"/>
+      <c r="A111" s="298"/>
+      <c r="B111" s="290" t="s">
+        <v>6</v>
+      </c>
+      <c r="C111" s="297">
+        <v>2</v>
+      </c>
+      <c r="D111" s="7">
+        <v>20000</v>
+      </c>
       <c r="E111" s="7">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="F111" s="298"/>
+        <f t="shared" si="6"/>
+        <v>40000</v>
+      </c>
+      <c r="F111" s="304"/>
     </row>
     <row r="112" s="249" customFormat="1" ht="14" customHeight="1" spans="1:6">
-      <c r="A112" s="291"/>
-      <c r="B112" s="290"/>
-      <c r="C112" s="297"/>
-      <c r="D112" s="7"/>
+      <c r="A112" s="298"/>
+      <c r="B112" s="290" t="s">
+        <v>10</v>
+      </c>
+      <c r="C112" s="297">
+        <v>0.3</v>
+      </c>
+      <c r="D112" s="7">
+        <v>20000</v>
+      </c>
       <c r="E112" s="7">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="F112" s="298"/>
+        <f t="shared" si="6"/>
+        <v>6000</v>
+      </c>
+      <c r="F112" s="304"/>
     </row>
     <row r="113" s="249" customFormat="1" ht="14" customHeight="1" spans="1:6">
-      <c r="A113" s="291"/>
-      <c r="B113" s="290"/>
-      <c r="C113" s="297"/>
-      <c r="D113" s="7"/>
+      <c r="A113" s="298"/>
+      <c r="B113" s="290" t="s">
+        <v>13</v>
+      </c>
+      <c r="C113" s="297">
+        <v>2</v>
+      </c>
+      <c r="D113" s="7">
+        <v>15000</v>
+      </c>
       <c r="E113" s="7">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="F113" s="298"/>
+        <f t="shared" si="6"/>
+        <v>30000</v>
+      </c>
+      <c r="F113" s="304"/>
     </row>
     <row r="114" s="249" customFormat="1" ht="14" customHeight="1" spans="1:6">
-      <c r="A114" s="291"/>
-      <c r="B114" s="290"/>
-      <c r="C114" s="297"/>
-      <c r="D114" s="7"/>
+      <c r="A114" s="298"/>
+      <c r="B114" s="290" t="s">
+        <v>36</v>
+      </c>
+      <c r="C114" s="297">
+        <v>2</v>
+      </c>
+      <c r="D114" s="7">
+        <v>48000</v>
+      </c>
       <c r="E114" s="7">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="F114" s="298"/>
+        <f t="shared" si="6"/>
+        <v>96000</v>
+      </c>
+      <c r="F114" s="304"/>
     </row>
     <row r="115" s="249" customFormat="1" ht="14" customHeight="1" spans="1:6">
-      <c r="A115" s="291"/>
-      <c r="B115" s="290"/>
-      <c r="C115" s="297"/>
-      <c r="D115" s="7"/>
+      <c r="A115" s="298"/>
+      <c r="B115" s="290" t="s">
+        <v>38</v>
+      </c>
+      <c r="C115" s="297">
+        <v>1</v>
+      </c>
+      <c r="D115" s="7">
+        <v>45000</v>
+      </c>
       <c r="E115" s="7">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="F115" s="298"/>
+        <f t="shared" si="6"/>
+        <v>45000</v>
+      </c>
+      <c r="F115" s="304"/>
     </row>
     <row r="116" s="249" customFormat="1" ht="14" customHeight="1" spans="1:6">
-      <c r="A116" s="291"/>
-      <c r="B116" s="290"/>
-      <c r="C116" s="297"/>
-      <c r="D116" s="7"/>
+      <c r="A116" s="298"/>
+      <c r="B116" s="290" t="s">
+        <v>11</v>
+      </c>
+      <c r="C116" s="297">
+        <v>1.2</v>
+      </c>
+      <c r="D116" s="7">
+        <v>38000</v>
+      </c>
       <c r="E116" s="7">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="F116" s="298"/>
+        <v>46000</v>
+      </c>
+      <c r="F116" s="304"/>
     </row>
     <row r="117" s="249" customFormat="1" ht="14" customHeight="1" spans="1:6">
-      <c r="A117" s="291"/>
-      <c r="B117" s="290"/>
-      <c r="C117" s="297"/>
-      <c r="D117" s="7"/>
+      <c r="A117" s="298"/>
+      <c r="B117" s="290" t="s">
+        <v>22</v>
+      </c>
+      <c r="C117" s="297">
+        <v>0.5</v>
+      </c>
+      <c r="D117" s="7">
+        <v>30000</v>
+      </c>
       <c r="E117" s="7">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="F117" s="298"/>
+        <f t="shared" si="6"/>
+        <v>15000</v>
+      </c>
+      <c r="F117" s="304"/>
     </row>
     <row r="118" s="249" customFormat="1" ht="14" customHeight="1" spans="1:6">
-      <c r="A118" s="291"/>
-      <c r="B118" s="290"/>
-      <c r="C118" s="297"/>
-      <c r="D118" s="7"/>
+      <c r="A118" s="298"/>
+      <c r="B118" s="290" t="s">
+        <v>14</v>
+      </c>
+      <c r="C118" s="297">
+        <v>3</v>
+      </c>
+      <c r="D118" s="7">
+        <v>24000</v>
+      </c>
       <c r="E118" s="7">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="F118" s="298"/>
+        <f t="shared" si="6"/>
+        <v>72000</v>
+      </c>
+      <c r="F118" s="304"/>
     </row>
     <row r="119" s="249" customFormat="1" ht="14" customHeight="1" spans="1:6">
-      <c r="A119" s="291"/>
-      <c r="B119" s="290"/>
-      <c r="C119" s="297"/>
-      <c r="D119" s="7"/>
+      <c r="A119" s="298"/>
+      <c r="B119" s="290" t="s">
+        <v>32</v>
+      </c>
+      <c r="C119" s="297">
+        <v>1</v>
+      </c>
+      <c r="D119" s="7">
+        <v>49000</v>
+      </c>
       <c r="E119" s="7">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="F119" s="298">
-        <f>SUM(E119:E134)</f>
-        <v>0</v>
-      </c>
+        <f t="shared" si="6"/>
+        <v>49000</v>
+      </c>
+      <c r="F119" s="304"/>
     </row>
     <row r="120" s="249" customFormat="1" ht="14" customHeight="1" spans="1:6">
-      <c r="A120" s="291"/>
-      <c r="B120" s="290"/>
-      <c r="C120" s="297"/>
-      <c r="D120" s="7"/>
+      <c r="A120" s="298"/>
+      <c r="B120" s="290" t="s">
+        <v>15</v>
+      </c>
+      <c r="C120" s="297">
+        <v>1</v>
+      </c>
+      <c r="D120" s="7">
+        <v>40000</v>
+      </c>
       <c r="E120" s="7">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="F120" s="298"/>
+        <f t="shared" si="6"/>
+        <v>40000</v>
+      </c>
+      <c r="F120" s="304"/>
     </row>
     <row r="121" s="249" customFormat="1" ht="14" customHeight="1" spans="1:6">
-      <c r="A121" s="291"/>
-      <c r="B121" s="290"/>
-      <c r="C121" s="297"/>
-      <c r="D121" s="7"/>
+      <c r="A121" s="300"/>
+      <c r="B121" s="290" t="s">
+        <v>27</v>
+      </c>
+      <c r="C121" s="297">
+        <v>5</v>
+      </c>
+      <c r="D121" s="7">
+        <v>20000</v>
+      </c>
       <c r="E121" s="7">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="F121" s="298"/>
+        <f t="shared" si="6"/>
+        <v>100000</v>
+      </c>
+      <c r="F121" s="305"/>
     </row>
     <row r="122" s="249" customFormat="1" ht="14" customHeight="1" spans="1:6">
       <c r="A122" s="291"/>
@@ -5491,10 +5654,10 @@
       <c r="C122" s="297"/>
       <c r="D122" s="7"/>
       <c r="E122" s="7">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="F122" s="298"/>
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="F122" s="306"/>
     </row>
     <row r="123" s="249" customFormat="1" ht="14" customHeight="1" spans="1:6">
       <c r="A123" s="291"/>
@@ -5502,10 +5665,10 @@
       <c r="C123" s="297"/>
       <c r="D123" s="7"/>
       <c r="E123" s="7">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="F123" s="298"/>
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="F123" s="306"/>
     </row>
     <row r="124" s="249" customFormat="1" ht="14" customHeight="1" spans="1:6">
       <c r="A124" s="291"/>
@@ -5513,10 +5676,10 @@
       <c r="C124" s="297"/>
       <c r="D124" s="7"/>
       <c r="E124" s="7">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="F124" s="298"/>
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="F124" s="306"/>
     </row>
     <row r="125" s="249" customFormat="1" ht="14" customHeight="1" spans="1:6">
       <c r="A125" s="291"/>
@@ -5524,10 +5687,10 @@
       <c r="C125" s="297"/>
       <c r="D125" s="7"/>
       <c r="E125" s="7">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="F125" s="298"/>
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="F125" s="306"/>
     </row>
     <row r="126" s="249" customFormat="1" ht="14" customHeight="1" spans="1:6">
       <c r="A126" s="291"/>
@@ -5535,10 +5698,10 @@
       <c r="C126" s="297"/>
       <c r="D126" s="7"/>
       <c r="E126" s="7">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="F126" s="298"/>
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="F126" s="306"/>
     </row>
     <row r="127" s="249" customFormat="1" ht="14" customHeight="1" spans="1:6">
       <c r="A127" s="291"/>
@@ -5546,10 +5709,10 @@
       <c r="C127" s="297"/>
       <c r="D127" s="7"/>
       <c r="E127" s="7">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="F127" s="298"/>
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="F127" s="306"/>
     </row>
     <row r="128" s="249" customFormat="1" ht="14" customHeight="1" spans="1:6">
       <c r="A128" s="291"/>
@@ -5557,10 +5720,13 @@
       <c r="C128" s="297"/>
       <c r="D128" s="7"/>
       <c r="E128" s="7">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="F128" s="298"/>
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="F128" s="306">
+        <f>SUM(E128:E143)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="129" s="249" customFormat="1" ht="14" customHeight="1" spans="1:6">
       <c r="A129" s="291"/>
@@ -5568,10 +5734,10 @@
       <c r="C129" s="297"/>
       <c r="D129" s="7"/>
       <c r="E129" s="7">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="F129" s="298"/>
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="F129" s="306"/>
     </row>
     <row r="130" s="249" customFormat="1" ht="14" customHeight="1" spans="1:6">
       <c r="A130" s="291"/>
@@ -5579,10 +5745,10 @@
       <c r="C130" s="297"/>
       <c r="D130" s="7"/>
       <c r="E130" s="7">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="F130" s="298"/>
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="F130" s="306"/>
     </row>
     <row r="131" s="249" customFormat="1" ht="14" customHeight="1" spans="1:6">
       <c r="A131" s="291"/>
@@ -5590,10 +5756,10 @@
       <c r="C131" s="297"/>
       <c r="D131" s="7"/>
       <c r="E131" s="7">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="F131" s="298"/>
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="F131" s="306"/>
     </row>
     <row r="132" s="249" customFormat="1" ht="14" customHeight="1" spans="1:6">
       <c r="A132" s="291"/>
@@ -5601,10 +5767,10 @@
       <c r="C132" s="297"/>
       <c r="D132" s="7"/>
       <c r="E132" s="7">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="F132" s="298"/>
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="F132" s="306"/>
     </row>
     <row r="133" s="249" customFormat="1" ht="14" customHeight="1" spans="1:6">
       <c r="A133" s="291"/>
@@ -5612,10 +5778,10 @@
       <c r="C133" s="297"/>
       <c r="D133" s="7"/>
       <c r="E133" s="7">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="F133" s="298"/>
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="F133" s="306"/>
     </row>
     <row r="134" s="249" customFormat="1" ht="14" customHeight="1" spans="1:6">
       <c r="A134" s="291"/>
@@ -5623,10 +5789,10 @@
       <c r="C134" s="297"/>
       <c r="D134" s="7"/>
       <c r="E134" s="7">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="F134" s="298"/>
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="F134" s="306"/>
     </row>
     <row r="135" s="249" customFormat="1" ht="14" customHeight="1" spans="1:6">
       <c r="A135" s="291"/>
@@ -5634,130 +5800,127 @@
       <c r="C135" s="297"/>
       <c r="D135" s="7"/>
       <c r="E135" s="7">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="F135" s="298">
-        <f>SUM(E135)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="136" s="249" customFormat="1" ht="14" customHeight="1" spans="1:7">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="F135" s="306"/>
+    </row>
+    <row r="136" s="249" customFormat="1" ht="14" customHeight="1" spans="1:6">
       <c r="A136" s="291"/>
       <c r="B136" s="290"/>
       <c r="C136" s="297"/>
       <c r="D136" s="7"/>
       <c r="E136" s="7">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="F136" s="298">
-        <f>SUM(E136:E140)</f>
-        <v>0</v>
-      </c>
-      <c r="G136" s="275"/>
-    </row>
-    <row r="137" s="249" customFormat="1" ht="17.6" spans="1:6">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="F136" s="306"/>
+    </row>
+    <row r="137" s="249" customFormat="1" ht="14" customHeight="1" spans="1:6">
       <c r="A137" s="291"/>
       <c r="B137" s="290"/>
       <c r="C137" s="297"/>
       <c r="D137" s="7"/>
       <c r="E137" s="7">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="F137" s="298"/>
-    </row>
-    <row r="138" s="249" customFormat="1" ht="17.6" spans="1:6">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="F137" s="306"/>
+    </row>
+    <row r="138" s="249" customFormat="1" ht="14" customHeight="1" spans="1:6">
       <c r="A138" s="291"/>
       <c r="B138" s="290"/>
       <c r="C138" s="297"/>
       <c r="D138" s="7"/>
       <c r="E138" s="7">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="F138" s="298"/>
-    </row>
-    <row r="139" s="249" customFormat="1" ht="17.6" spans="1:6">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="F138" s="306"/>
+    </row>
+    <row r="139" s="249" customFormat="1" ht="14" customHeight="1" spans="1:6">
       <c r="A139" s="291"/>
       <c r="B139" s="290"/>
       <c r="C139" s="297"/>
       <c r="D139" s="7"/>
       <c r="E139" s="7">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="F139" s="298"/>
-    </row>
-    <row r="140" s="249" customFormat="1" ht="17.6" spans="1:6">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="F139" s="306"/>
+    </row>
+    <row r="140" s="249" customFormat="1" ht="14" customHeight="1" spans="1:6">
       <c r="A140" s="291"/>
       <c r="B140" s="290"/>
       <c r="C140" s="297"/>
       <c r="D140" s="7"/>
       <c r="E140" s="7">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="F140" s="298"/>
-    </row>
-    <row r="141" s="249" customFormat="1" ht="17.6" spans="1:6">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="F140" s="306"/>
+    </row>
+    <row r="141" s="249" customFormat="1" ht="14" customHeight="1" spans="1:6">
       <c r="A141" s="291"/>
-      <c r="B141" s="299"/>
-      <c r="C141" s="300"/>
-      <c r="D141" s="134"/>
+      <c r="B141" s="290"/>
+      <c r="C141" s="297"/>
+      <c r="D141" s="7"/>
       <c r="E141" s="7">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="F141" s="298">
-        <f>SUM(E141:E147)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="142" s="249" customFormat="1" ht="17.6" spans="1:6">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="F141" s="306"/>
+    </row>
+    <row r="142" s="249" customFormat="1" ht="14" customHeight="1" spans="1:6">
       <c r="A142" s="291"/>
       <c r="B142" s="290"/>
       <c r="C142" s="297"/>
       <c r="D142" s="7"/>
       <c r="E142" s="7">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="F142" s="298"/>
-    </row>
-    <row r="143" s="249" customFormat="1" ht="17.6" spans="1:6">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="F142" s="306"/>
+    </row>
+    <row r="143" s="249" customFormat="1" ht="14" customHeight="1" spans="1:6">
       <c r="A143" s="291"/>
       <c r="B143" s="290"/>
       <c r="C143" s="297"/>
       <c r="D143" s="7"/>
       <c r="E143" s="7">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="F143" s="298"/>
-    </row>
-    <row r="144" s="249" customFormat="1" ht="17.6" spans="1:6">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="F143" s="306"/>
+    </row>
+    <row r="144" s="249" customFormat="1" ht="14" customHeight="1" spans="1:6">
       <c r="A144" s="291"/>
       <c r="B144" s="290"/>
       <c r="C144" s="297"/>
       <c r="D144" s="7"/>
       <c r="E144" s="7">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="F144" s="298"/>
-    </row>
-    <row r="145" s="249" customFormat="1" ht="17.6" spans="1:6">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="F144" s="306">
+        <f>SUM(E144)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="145" s="249" customFormat="1" ht="14" customHeight="1" spans="1:7">
       <c r="A145" s="291"/>
       <c r="B145" s="290"/>
       <c r="C145" s="297"/>
       <c r="D145" s="7"/>
       <c r="E145" s="7">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="F145" s="298"/>
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="F145" s="306">
+        <f>SUM(E145:E149)</f>
+        <v>0</v>
+      </c>
+      <c r="G145" s="275"/>
     </row>
     <row r="146" s="249" customFormat="1" ht="17.6" spans="1:6">
       <c r="A146" s="291"/>
@@ -5765,21 +5928,21 @@
       <c r="C146" s="297"/>
       <c r="D146" s="7"/>
       <c r="E146" s="7">
-        <f t="shared" ref="E146:E209" si="6">SUM(C146*D146)</f>
-        <v>0</v>
-      </c>
-      <c r="F146" s="298"/>
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="F146" s="306"/>
     </row>
     <row r="147" s="249" customFormat="1" ht="17.6" spans="1:6">
       <c r="A147" s="291"/>
       <c r="B147" s="290"/>
       <c r="C147" s="297"/>
-      <c r="D147" s="266"/>
+      <c r="D147" s="7"/>
       <c r="E147" s="7">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="F147" s="298"/>
+      <c r="F147" s="306"/>
     </row>
     <row r="148" s="249" customFormat="1" ht="17.6" spans="1:6">
       <c r="A148" s="291"/>
@@ -5790,10 +5953,7 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="F148" s="298">
-        <f>SUM(E148:E155)</f>
-        <v>0</v>
-      </c>
+      <c r="F148" s="306"/>
     </row>
     <row r="149" s="249" customFormat="1" ht="17.6" spans="1:6">
       <c r="A149" s="291"/>
@@ -5804,18 +5964,21 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="F149" s="298"/>
+      <c r="F149" s="306"/>
     </row>
     <row r="150" s="249" customFormat="1" ht="17.6" spans="1:6">
       <c r="A150" s="291"/>
-      <c r="B150" s="290"/>
-      <c r="C150" s="297"/>
-      <c r="D150" s="7"/>
+      <c r="B150" s="307"/>
+      <c r="C150" s="308"/>
+      <c r="D150" s="134"/>
       <c r="E150" s="7">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="F150" s="298"/>
+      <c r="F150" s="306">
+        <f>SUM(E150:E156)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="151" s="249" customFormat="1" ht="17.6" spans="1:6">
       <c r="A151" s="291"/>
@@ -5826,7 +5989,7 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="F151" s="298"/>
+      <c r="F151" s="306"/>
     </row>
     <row r="152" s="249" customFormat="1" ht="17.6" spans="1:6">
       <c r="A152" s="291"/>
@@ -5837,7 +6000,7 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="F152" s="298"/>
+      <c r="F152" s="306"/>
     </row>
     <row r="153" s="249" customFormat="1" ht="17.6" spans="1:6">
       <c r="A153" s="291"/>
@@ -5848,7 +6011,7 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="F153" s="298"/>
+      <c r="F153" s="306"/>
     </row>
     <row r="154" s="249" customFormat="1" ht="17.6" spans="1:6">
       <c r="A154" s="291"/>
@@ -5859,7 +6022,7 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="F154" s="298"/>
+      <c r="F154" s="306"/>
     </row>
     <row r="155" s="249" customFormat="1" ht="17.6" spans="1:6">
       <c r="A155" s="291"/>
@@ -5867,24 +6030,21 @@
       <c r="C155" s="297"/>
       <c r="D155" s="7"/>
       <c r="E155" s="7">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="F155" s="298"/>
+        <f t="shared" ref="E155:E218" si="7">SUM(C155*D155)</f>
+        <v>0</v>
+      </c>
+      <c r="F155" s="306"/>
     </row>
     <row r="156" s="249" customFormat="1" ht="17.6" spans="1:6">
       <c r="A156" s="291"/>
       <c r="B156" s="290"/>
       <c r="C156" s="297"/>
-      <c r="D156" s="7"/>
+      <c r="D156" s="266"/>
       <c r="E156" s="7">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="F156" s="298">
-        <f>SUM(E156:E162)</f>
-        <v>0</v>
-      </c>
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="F156" s="306"/>
     </row>
     <row r="157" s="249" customFormat="1" ht="17.6" spans="1:6">
       <c r="A157" s="291"/>
@@ -5892,10 +6052,13 @@
       <c r="C157" s="297"/>
       <c r="D157" s="7"/>
       <c r="E157" s="7">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="F157" s="298"/>
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="F157" s="306">
+        <f>SUM(E157:E164)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="158" s="249" customFormat="1" ht="17.6" spans="1:6">
       <c r="A158" s="291"/>
@@ -5903,10 +6066,10 @@
       <c r="C158" s="297"/>
       <c r="D158" s="7"/>
       <c r="E158" s="7">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="F158" s="298"/>
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="F158" s="306"/>
     </row>
     <row r="159" s="249" customFormat="1" ht="17.6" spans="1:6">
       <c r="A159" s="291"/>
@@ -5914,10 +6077,10 @@
       <c r="C159" s="297"/>
       <c r="D159" s="7"/>
       <c r="E159" s="7">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="F159" s="298"/>
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="F159" s="306"/>
     </row>
     <row r="160" s="249" customFormat="1" ht="17.6" spans="1:6">
       <c r="A160" s="291"/>
@@ -5925,10 +6088,10 @@
       <c r="C160" s="297"/>
       <c r="D160" s="7"/>
       <c r="E160" s="7">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="F160" s="298"/>
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="F160" s="306"/>
     </row>
     <row r="161" s="249" customFormat="1" ht="17.6" spans="1:6">
       <c r="A161" s="291"/>
@@ -5936,10 +6099,10 @@
       <c r="C161" s="297"/>
       <c r="D161" s="7"/>
       <c r="E161" s="7">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="F161" s="298"/>
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="F161" s="306"/>
     </row>
     <row r="162" s="249" customFormat="1" ht="17.6" spans="1:6">
       <c r="A162" s="291"/>
@@ -5947,10 +6110,10 @@
       <c r="C162" s="297"/>
       <c r="D162" s="7"/>
       <c r="E162" s="7">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="F162" s="298"/>
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="F162" s="306"/>
     </row>
     <row r="163" s="249" customFormat="1" ht="17.6" spans="1:6">
       <c r="A163" s="291"/>
@@ -5958,13 +6121,10 @@
       <c r="C163" s="297"/>
       <c r="D163" s="7"/>
       <c r="E163" s="7">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="F163" s="298">
-        <f>SUM(E163:E172)</f>
-        <v>0</v>
-      </c>
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="F163" s="306"/>
     </row>
     <row r="164" s="249" customFormat="1" ht="17.6" spans="1:6">
       <c r="A164" s="291"/>
@@ -5972,10 +6132,10 @@
       <c r="C164" s="297"/>
       <c r="D164" s="7"/>
       <c r="E164" s="7">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="F164" s="298"/>
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="F164" s="306"/>
     </row>
     <row r="165" s="249" customFormat="1" ht="17.6" spans="1:6">
       <c r="A165" s="291"/>
@@ -5983,10 +6143,13 @@
       <c r="C165" s="297"/>
       <c r="D165" s="7"/>
       <c r="E165" s="7">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="F165" s="298"/>
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="F165" s="306">
+        <f>SUM(E165:E171)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="166" s="249" customFormat="1" ht="17.6" spans="1:6">
       <c r="A166" s="291"/>
@@ -5994,10 +6157,10 @@
       <c r="C166" s="297"/>
       <c r="D166" s="7"/>
       <c r="E166" s="7">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="F166" s="298"/>
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="F166" s="306"/>
     </row>
     <row r="167" s="249" customFormat="1" ht="17.6" spans="1:6">
       <c r="A167" s="291"/>
@@ -6005,10 +6168,10 @@
       <c r="C167" s="297"/>
       <c r="D167" s="7"/>
       <c r="E167" s="7">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="F167" s="298"/>
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="F167" s="306"/>
     </row>
     <row r="168" s="249" customFormat="1" ht="17.6" spans="1:6">
       <c r="A168" s="291"/>
@@ -6016,10 +6179,10 @@
       <c r="C168" s="297"/>
       <c r="D168" s="7"/>
       <c r="E168" s="7">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="F168" s="298"/>
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="F168" s="306"/>
     </row>
     <row r="169" s="249" customFormat="1" ht="17.6" spans="1:6">
       <c r="A169" s="291"/>
@@ -6027,10 +6190,10 @@
       <c r="C169" s="297"/>
       <c r="D169" s="7"/>
       <c r="E169" s="7">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="F169" s="298"/>
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="F169" s="306"/>
     </row>
     <row r="170" s="249" customFormat="1" ht="17.6" spans="1:6">
       <c r="A170" s="291"/>
@@ -6038,10 +6201,10 @@
       <c r="C170" s="297"/>
       <c r="D170" s="7"/>
       <c r="E170" s="7">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="F170" s="298"/>
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="F170" s="306"/>
     </row>
     <row r="171" s="249" customFormat="1" ht="17.6" spans="1:6">
       <c r="A171" s="291"/>
@@ -6049,10 +6212,10 @@
       <c r="C171" s="297"/>
       <c r="D171" s="7"/>
       <c r="E171" s="7">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="F171" s="298"/>
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="F171" s="306"/>
     </row>
     <row r="172" s="249" customFormat="1" ht="17.6" spans="1:6">
       <c r="A172" s="291"/>
@@ -6060,10 +6223,13 @@
       <c r="C172" s="297"/>
       <c r="D172" s="7"/>
       <c r="E172" s="7">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="F172" s="298"/>
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="F172" s="306">
+        <f>SUM(E172:E181)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="173" s="249" customFormat="1" ht="17.6" spans="1:6">
       <c r="A173" s="291"/>
@@ -6071,13 +6237,10 @@
       <c r="C173" s="297"/>
       <c r="D173" s="7"/>
       <c r="E173" s="7">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="F173" s="298">
-        <f>SUM(E173:E186)</f>
-        <v>0</v>
-      </c>
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="F173" s="306"/>
     </row>
     <row r="174" s="249" customFormat="1" ht="17.6" spans="1:6">
       <c r="A174" s="291"/>
@@ -6085,10 +6248,10 @@
       <c r="C174" s="297"/>
       <c r="D174" s="7"/>
       <c r="E174" s="7">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="F174" s="298"/>
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="F174" s="306"/>
     </row>
     <row r="175" s="249" customFormat="1" ht="17.6" spans="1:6">
       <c r="A175" s="291"/>
@@ -6096,10 +6259,10 @@
       <c r="C175" s="297"/>
       <c r="D175" s="7"/>
       <c r="E175" s="7">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="F175" s="298"/>
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="F175" s="306"/>
     </row>
     <row r="176" s="249" customFormat="1" ht="17.6" spans="1:6">
       <c r="A176" s="291"/>
@@ -6107,10 +6270,10 @@
       <c r="C176" s="297"/>
       <c r="D176" s="7"/>
       <c r="E176" s="7">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="F176" s="298"/>
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="F176" s="306"/>
     </row>
     <row r="177" s="249" customFormat="1" ht="17.6" spans="1:6">
       <c r="A177" s="291"/>
@@ -6118,10 +6281,10 @@
       <c r="C177" s="297"/>
       <c r="D177" s="7"/>
       <c r="E177" s="7">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="F177" s="298"/>
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="F177" s="306"/>
     </row>
     <row r="178" s="249" customFormat="1" ht="17.6" spans="1:6">
       <c r="A178" s="291"/>
@@ -6129,10 +6292,10 @@
       <c r="C178" s="297"/>
       <c r="D178" s="7"/>
       <c r="E178" s="7">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="F178" s="298"/>
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="F178" s="306"/>
     </row>
     <row r="179" s="249" customFormat="1" ht="17.6" spans="1:6">
       <c r="A179" s="291"/>
@@ -6140,10 +6303,10 @@
       <c r="C179" s="297"/>
       <c r="D179" s="7"/>
       <c r="E179" s="7">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="F179" s="298"/>
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="F179" s="306"/>
     </row>
     <row r="180" s="249" customFormat="1" ht="17.6" spans="1:6">
       <c r="A180" s="291"/>
@@ -6151,10 +6314,10 @@
       <c r="C180" s="297"/>
       <c r="D180" s="7"/>
       <c r="E180" s="7">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="F180" s="298"/>
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="F180" s="306"/>
     </row>
     <row r="181" s="249" customFormat="1" ht="17.6" spans="1:6">
       <c r="A181" s="291"/>
@@ -6162,10 +6325,10 @@
       <c r="C181" s="297"/>
       <c r="D181" s="7"/>
       <c r="E181" s="7">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="F181" s="298"/>
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="F181" s="306"/>
     </row>
     <row r="182" s="249" customFormat="1" ht="17.6" spans="1:6">
       <c r="A182" s="291"/>
@@ -6173,10 +6336,13 @@
       <c r="C182" s="297"/>
       <c r="D182" s="7"/>
       <c r="E182" s="7">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="F182" s="298"/>
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="F182" s="306">
+        <f>SUM(E182:E195)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="183" s="249" customFormat="1" ht="17.6" spans="1:6">
       <c r="A183" s="291"/>
@@ -6184,10 +6350,10 @@
       <c r="C183" s="297"/>
       <c r="D183" s="7"/>
       <c r="E183" s="7">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="F183" s="298"/>
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="F183" s="306"/>
     </row>
     <row r="184" s="249" customFormat="1" ht="17.6" spans="1:6">
       <c r="A184" s="291"/>
@@ -6195,10 +6361,10 @@
       <c r="C184" s="297"/>
       <c r="D184" s="7"/>
       <c r="E184" s="7">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="F184" s="298"/>
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="F184" s="306"/>
     </row>
     <row r="185" s="249" customFormat="1" ht="17.6" spans="1:6">
       <c r="A185" s="291"/>
@@ -6206,10 +6372,10 @@
       <c r="C185" s="297"/>
       <c r="D185" s="7"/>
       <c r="E185" s="7">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="F185" s="298"/>
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="F185" s="306"/>
     </row>
     <row r="186" s="249" customFormat="1" ht="17.6" spans="1:6">
       <c r="A186" s="291"/>
@@ -6217,10 +6383,10 @@
       <c r="C186" s="297"/>
       <c r="D186" s="7"/>
       <c r="E186" s="7">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="F186" s="298"/>
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="F186" s="306"/>
     </row>
     <row r="187" s="249" customFormat="1" ht="17.6" spans="1:6">
       <c r="A187" s="291"/>
@@ -6228,13 +6394,10 @@
       <c r="C187" s="297"/>
       <c r="D187" s="7"/>
       <c r="E187" s="7">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="F187" s="298">
-        <f>SUM(E187)</f>
-        <v>0</v>
-      </c>
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="F187" s="306"/>
     </row>
     <row r="188" s="249" customFormat="1" ht="17.6" spans="1:6">
       <c r="A188" s="291"/>
@@ -6242,13 +6405,10 @@
       <c r="C188" s="297"/>
       <c r="D188" s="7"/>
       <c r="E188" s="7">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="F188" s="298">
-        <f>SUM(E188:E203)</f>
-        <v>0</v>
-      </c>
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="F188" s="306"/>
     </row>
     <row r="189" s="249" customFormat="1" ht="17.6" spans="1:6">
       <c r="A189" s="291"/>
@@ -6256,10 +6416,10 @@
       <c r="C189" s="297"/>
       <c r="D189" s="7"/>
       <c r="E189" s="7">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="F189" s="298"/>
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="F189" s="306"/>
     </row>
     <row r="190" s="249" customFormat="1" ht="17.6" spans="1:6">
       <c r="A190" s="291"/>
@@ -6267,10 +6427,10 @@
       <c r="C190" s="297"/>
       <c r="D190" s="7"/>
       <c r="E190" s="7">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="F190" s="298"/>
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="F190" s="306"/>
     </row>
     <row r="191" s="249" customFormat="1" ht="17.6" spans="1:6">
       <c r="A191" s="291"/>
@@ -6278,10 +6438,10 @@
       <c r="C191" s="297"/>
       <c r="D191" s="7"/>
       <c r="E191" s="7">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="F191" s="298"/>
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="F191" s="306"/>
     </row>
     <row r="192" s="249" customFormat="1" ht="17.6" spans="1:6">
       <c r="A192" s="291"/>
@@ -6289,10 +6449,10 @@
       <c r="C192" s="297"/>
       <c r="D192" s="7"/>
       <c r="E192" s="7">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="F192" s="298"/>
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="F192" s="306"/>
     </row>
     <row r="193" s="249" customFormat="1" ht="17.6" spans="1:6">
       <c r="A193" s="291"/>
@@ -6300,10 +6460,10 @@
       <c r="C193" s="297"/>
       <c r="D193" s="7"/>
       <c r="E193" s="7">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="F193" s="298"/>
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="F193" s="306"/>
     </row>
     <row r="194" s="249" customFormat="1" ht="17.6" spans="1:6">
       <c r="A194" s="291"/>
@@ -6311,10 +6471,10 @@
       <c r="C194" s="297"/>
       <c r="D194" s="7"/>
       <c r="E194" s="7">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="F194" s="298"/>
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="F194" s="306"/>
     </row>
     <row r="195" s="249" customFormat="1" ht="17.6" spans="1:6">
       <c r="A195" s="291"/>
@@ -6322,10 +6482,10 @@
       <c r="C195" s="297"/>
       <c r="D195" s="7"/>
       <c r="E195" s="7">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="F195" s="298"/>
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="F195" s="306"/>
     </row>
     <row r="196" s="249" customFormat="1" ht="17.6" spans="1:6">
       <c r="A196" s="291"/>
@@ -6333,10 +6493,13 @@
       <c r="C196" s="297"/>
       <c r="D196" s="7"/>
       <c r="E196" s="7">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="F196" s="298"/>
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="F196" s="306">
+        <f>SUM(E196)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="197" s="249" customFormat="1" ht="17.6" spans="1:6">
       <c r="A197" s="291"/>
@@ -6344,10 +6507,13 @@
       <c r="C197" s="297"/>
       <c r="D197" s="7"/>
       <c r="E197" s="7">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="F197" s="298"/>
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="F197" s="306">
+        <f>SUM(E197:E212)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="198" s="249" customFormat="1" ht="17.6" spans="1:6">
       <c r="A198" s="291"/>
@@ -6355,10 +6521,10 @@
       <c r="C198" s="297"/>
       <c r="D198" s="7"/>
       <c r="E198" s="7">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="F198" s="298"/>
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="F198" s="306"/>
     </row>
     <row r="199" s="249" customFormat="1" ht="17.6" spans="1:6">
       <c r="A199" s="291"/>
@@ -6366,10 +6532,10 @@
       <c r="C199" s="297"/>
       <c r="D199" s="7"/>
       <c r="E199" s="7">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="F199" s="298"/>
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="F199" s="306"/>
     </row>
     <row r="200" s="249" customFormat="1" ht="17.6" spans="1:6">
       <c r="A200" s="291"/>
@@ -6377,10 +6543,10 @@
       <c r="C200" s="297"/>
       <c r="D200" s="7"/>
       <c r="E200" s="7">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="F200" s="298"/>
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="F200" s="306"/>
     </row>
     <row r="201" s="249" customFormat="1" ht="17.6" spans="1:6">
       <c r="A201" s="291"/>
@@ -6388,21 +6554,21 @@
       <c r="C201" s="297"/>
       <c r="D201" s="7"/>
       <c r="E201" s="7">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="F201" s="298"/>
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="F201" s="306"/>
     </row>
     <row r="202" s="249" customFormat="1" ht="17.6" spans="1:6">
       <c r="A202" s="291"/>
-      <c r="B202" s="299"/>
-      <c r="C202" s="300"/>
-      <c r="D202" s="134"/>
+      <c r="B202" s="290"/>
+      <c r="C202" s="297"/>
+      <c r="D202" s="7"/>
       <c r="E202" s="7">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="F202" s="298"/>
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="F202" s="306"/>
     </row>
     <row r="203" s="249" customFormat="1" ht="17.6" spans="1:6">
       <c r="A203" s="291"/>
@@ -6410,104 +6576,101 @@
       <c r="C203" s="297"/>
       <c r="D203" s="7"/>
       <c r="E203" s="7">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="F203" s="298"/>
-    </row>
-    <row r="204" s="249" customFormat="1" spans="1:6">
-      <c r="A204" s="283"/>
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="F203" s="306"/>
+    </row>
+    <row r="204" s="249" customFormat="1" ht="17.6" spans="1:6">
+      <c r="A204" s="291"/>
       <c r="B204" s="290"/>
       <c r="C204" s="297"/>
       <c r="D204" s="7"/>
       <c r="E204" s="7">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="F204" s="293">
-        <f>SUM(E204:E211)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="205" s="249" customFormat="1" spans="1:6">
-      <c r="A205" s="286"/>
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="F204" s="306"/>
+    </row>
+    <row r="205" s="249" customFormat="1" ht="17.6" spans="1:6">
+      <c r="A205" s="291"/>
       <c r="B205" s="290"/>
       <c r="C205" s="297"/>
       <c r="D205" s="7"/>
       <c r="E205" s="7">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="F205" s="294"/>
-    </row>
-    <row r="206" s="249" customFormat="1" spans="1:6">
-      <c r="A206" s="286"/>
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="F205" s="306"/>
+    </row>
+    <row r="206" s="249" customFormat="1" ht="17.6" spans="1:6">
+      <c r="A206" s="291"/>
       <c r="B206" s="290"/>
       <c r="C206" s="297"/>
       <c r="D206" s="7"/>
       <c r="E206" s="7">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="F206" s="294"/>
-    </row>
-    <row r="207" s="249" customFormat="1" spans="1:6">
-      <c r="A207" s="286"/>
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="F206" s="306"/>
+    </row>
+    <row r="207" s="249" customFormat="1" ht="17.6" spans="1:6">
+      <c r="A207" s="291"/>
       <c r="B207" s="290"/>
       <c r="C207" s="297"/>
       <c r="D207" s="7"/>
       <c r="E207" s="7">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="F207" s="294"/>
-    </row>
-    <row r="208" s="249" customFormat="1" spans="1:6">
-      <c r="A208" s="286"/>
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="F207" s="306"/>
+    </row>
+    <row r="208" s="249" customFormat="1" ht="17.6" spans="1:6">
+      <c r="A208" s="291"/>
       <c r="B208" s="290"/>
       <c r="C208" s="297"/>
       <c r="D208" s="7"/>
       <c r="E208" s="7">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="F208" s="294"/>
-    </row>
-    <row r="209" s="249" customFormat="1" spans="1:6">
-      <c r="A209" s="286"/>
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="F208" s="306"/>
+    </row>
+    <row r="209" s="249" customFormat="1" ht="17.6" spans="1:6">
+      <c r="A209" s="291"/>
       <c r="B209" s="290"/>
       <c r="C209" s="297"/>
       <c r="D209" s="7"/>
       <c r="E209" s="7">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="F209" s="294"/>
-    </row>
-    <row r="210" s="249" customFormat="1" spans="1:6">
-      <c r="A210" s="286"/>
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="F209" s="306"/>
+    </row>
+    <row r="210" s="249" customFormat="1" ht="17.6" spans="1:6">
+      <c r="A210" s="291"/>
       <c r="B210" s="290"/>
       <c r="C210" s="297"/>
       <c r="D210" s="7"/>
       <c r="E210" s="7">
-        <f t="shared" ref="E210:E273" si="7">SUM(C210*D210)</f>
-        <v>0</v>
-      </c>
-      <c r="F210" s="294"/>
-    </row>
-    <row r="211" s="249" customFormat="1" spans="1:6">
-      <c r="A211" s="287"/>
-      <c r="B211" s="290"/>
-      <c r="C211" s="297"/>
-      <c r="D211" s="7"/>
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="F210" s="306"/>
+    </row>
+    <row r="211" s="249" customFormat="1" ht="17.6" spans="1:6">
+      <c r="A211" s="291"/>
+      <c r="B211" s="307"/>
+      <c r="C211" s="308"/>
+      <c r="D211" s="134"/>
       <c r="E211" s="7">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="F211" s="295"/>
-    </row>
-    <row r="212" s="249" customFormat="1" spans="1:6">
-      <c r="A212" s="283"/>
+      <c r="F211" s="306"/>
+    </row>
+    <row r="212" s="249" customFormat="1" ht="17.6" spans="1:6">
+      <c r="A212" s="291"/>
       <c r="B212" s="290"/>
       <c r="C212" s="297"/>
       <c r="D212" s="7"/>
@@ -6515,13 +6678,10 @@
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="F212" s="293">
-        <f>SUM(E212:E223)</f>
-        <v>0</v>
-      </c>
+      <c r="F212" s="306"/>
     </row>
     <row r="213" s="249" customFormat="1" spans="1:6">
-      <c r="A213" s="286"/>
+      <c r="A213" s="283"/>
       <c r="B213" s="290"/>
       <c r="C213" s="297"/>
       <c r="D213" s="7"/>
@@ -6529,7 +6689,10 @@
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="F213" s="294"/>
+      <c r="F213" s="293">
+        <f>SUM(E213:E220)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="214" s="249" customFormat="1" spans="1:6">
       <c r="A214" s="286"/>
@@ -6592,32 +6755,35 @@
       <c r="C219" s="297"/>
       <c r="D219" s="7"/>
       <c r="E219" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" ref="E219:E282" si="8">SUM(C219*D219)</f>
         <v>0</v>
       </c>
       <c r="F219" s="294"/>
     </row>
     <row r="220" s="249" customFormat="1" spans="1:6">
-      <c r="A220" s="286"/>
+      <c r="A220" s="287"/>
       <c r="B220" s="290"/>
       <c r="C220" s="297"/>
       <c r="D220" s="7"/>
       <c r="E220" s="7">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="F220" s="294"/>
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="F220" s="295"/>
     </row>
     <row r="221" s="249" customFormat="1" spans="1:6">
-      <c r="A221" s="286"/>
+      <c r="A221" s="283"/>
       <c r="B221" s="290"/>
       <c r="C221" s="297"/>
       <c r="D221" s="7"/>
       <c r="E221" s="7">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="F221" s="294"/>
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="F221" s="293">
+        <f>SUM(E221:E232)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="222" s="249" customFormat="1" spans="1:6">
       <c r="A222" s="286"/>
@@ -6625,35 +6791,32 @@
       <c r="C222" s="297"/>
       <c r="D222" s="7"/>
       <c r="E222" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="F222" s="294"/>
     </row>
     <row r="223" s="249" customFormat="1" spans="1:6">
-      <c r="A223" s="287"/>
+      <c r="A223" s="286"/>
       <c r="B223" s="290"/>
       <c r="C223" s="297"/>
       <c r="D223" s="7"/>
       <c r="E223" s="7">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="F223" s="295"/>
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="F223" s="294"/>
     </row>
     <row r="224" s="249" customFormat="1" spans="1:6">
-      <c r="A224" s="283"/>
+      <c r="A224" s="286"/>
       <c r="B224" s="290"/>
       <c r="C224" s="297"/>
       <c r="D224" s="7"/>
       <c r="E224" s="7">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="F224" s="293">
-        <f>SUM(E224:E232)</f>
-        <v>0</v>
-      </c>
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="F224" s="294"/>
     </row>
     <row r="225" s="249" customFormat="1" spans="1:6">
       <c r="A225" s="286"/>
@@ -6661,7 +6824,7 @@
       <c r="C225" s="297"/>
       <c r="D225" s="7"/>
       <c r="E225" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="F225" s="294"/>
@@ -6672,7 +6835,7 @@
       <c r="C226" s="297"/>
       <c r="D226" s="7"/>
       <c r="E226" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="F226" s="294"/>
@@ -6683,7 +6846,7 @@
       <c r="C227" s="297"/>
       <c r="D227" s="7"/>
       <c r="E227" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="F227" s="294"/>
@@ -6694,7 +6857,7 @@
       <c r="C228" s="297"/>
       <c r="D228" s="7"/>
       <c r="E228" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="F228" s="294"/>
@@ -6705,7 +6868,7 @@
       <c r="C229" s="297"/>
       <c r="D229" s="7"/>
       <c r="E229" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="F229" s="294"/>
@@ -6716,7 +6879,7 @@
       <c r="C230" s="297"/>
       <c r="D230" s="7"/>
       <c r="E230" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="F230" s="294"/>
@@ -6727,7 +6890,7 @@
       <c r="C231" s="297"/>
       <c r="D231" s="7"/>
       <c r="E231" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="F231" s="294"/>
@@ -6738,7 +6901,7 @@
       <c r="C232" s="297"/>
       <c r="D232" s="7"/>
       <c r="E232" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="F232" s="295"/>
@@ -6749,11 +6912,11 @@
       <c r="C233" s="297"/>
       <c r="D233" s="7"/>
       <c r="E233" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="F233" s="293">
-        <f>SUM(E233:E243)</f>
+        <f>SUM(E233:E241)</f>
         <v>0</v>
       </c>
     </row>
@@ -6763,7 +6926,7 @@
       <c r="C234" s="297"/>
       <c r="D234" s="7"/>
       <c r="E234" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="F234" s="294"/>
@@ -6774,7 +6937,7 @@
       <c r="C235" s="297"/>
       <c r="D235" s="7"/>
       <c r="E235" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="F235" s="294"/>
@@ -6785,7 +6948,7 @@
       <c r="C236" s="297"/>
       <c r="D236" s="7"/>
       <c r="E236" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="F236" s="294"/>
@@ -6796,7 +6959,7 @@
       <c r="C237" s="297"/>
       <c r="D237" s="7"/>
       <c r="E237" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="F237" s="294"/>
@@ -6807,7 +6970,7 @@
       <c r="C238" s="297"/>
       <c r="D238" s="7"/>
       <c r="E238" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="F238" s="294"/>
@@ -6818,7 +6981,7 @@
       <c r="C239" s="297"/>
       <c r="D239" s="7"/>
       <c r="E239" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="F239" s="294"/>
@@ -6829,57 +6992,57 @@
       <c r="C240" s="297"/>
       <c r="D240" s="7"/>
       <c r="E240" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="F240" s="294"/>
     </row>
     <row r="241" s="249" customFormat="1" spans="1:6">
-      <c r="A241" s="286"/>
+      <c r="A241" s="287"/>
       <c r="B241" s="290"/>
       <c r="C241" s="297"/>
       <c r="D241" s="7"/>
       <c r="E241" s="7">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="F241" s="294"/>
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="F241" s="295"/>
     </row>
     <row r="242" s="249" customFormat="1" spans="1:6">
-      <c r="A242" s="286"/>
+      <c r="A242" s="283"/>
       <c r="B242" s="290"/>
       <c r="C242" s="297"/>
       <c r="D242" s="7"/>
       <c r="E242" s="7">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="F242" s="294"/>
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="F242" s="293">
+        <f>SUM(E242:E252)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="243" s="249" customFormat="1" spans="1:6">
-      <c r="A243" s="287"/>
+      <c r="A243" s="286"/>
       <c r="B243" s="290"/>
       <c r="C243" s="297"/>
       <c r="D243" s="7"/>
       <c r="E243" s="7">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="F243" s="295"/>
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="F243" s="294"/>
     </row>
     <row r="244" s="249" customFormat="1" spans="1:6">
-      <c r="A244" s="283"/>
+      <c r="A244" s="286"/>
       <c r="B244" s="290"/>
       <c r="C244" s="297"/>
       <c r="D244" s="7"/>
       <c r="E244" s="7">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="F244" s="293">
-        <f>SUM(E244:E254)</f>
-        <v>0</v>
-      </c>
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="F244" s="294"/>
     </row>
     <row r="245" s="249" customFormat="1" spans="1:6">
       <c r="A245" s="286"/>
@@ -6887,7 +7050,7 @@
       <c r="C245" s="297"/>
       <c r="D245" s="7"/>
       <c r="E245" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="F245" s="294"/>
@@ -6898,7 +7061,7 @@
       <c r="C246" s="297"/>
       <c r="D246" s="7"/>
       <c r="E246" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="F246" s="294"/>
@@ -6909,7 +7072,7 @@
       <c r="C247" s="297"/>
       <c r="D247" s="7"/>
       <c r="E247" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="F247" s="294"/>
@@ -6920,7 +7083,7 @@
       <c r="C248" s="297"/>
       <c r="D248" s="7"/>
       <c r="E248" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="F248" s="294"/>
@@ -6931,7 +7094,7 @@
       <c r="C249" s="297"/>
       <c r="D249" s="7"/>
       <c r="E249" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="F249" s="294"/>
@@ -6942,7 +7105,7 @@
       <c r="C250" s="297"/>
       <c r="D250" s="7"/>
       <c r="E250" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="F250" s="294"/>
@@ -6953,57 +7116,57 @@
       <c r="C251" s="297"/>
       <c r="D251" s="7"/>
       <c r="E251" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="F251" s="294"/>
     </row>
     <row r="252" s="249" customFormat="1" spans="1:6">
-      <c r="A252" s="286"/>
+      <c r="A252" s="287"/>
       <c r="B252" s="290"/>
       <c r="C252" s="297"/>
       <c r="D252" s="7"/>
       <c r="E252" s="7">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="F252" s="294"/>
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="F252" s="295"/>
     </row>
     <row r="253" s="249" customFormat="1" spans="1:6">
-      <c r="A253" s="286"/>
+      <c r="A253" s="283"/>
       <c r="B253" s="290"/>
       <c r="C253" s="297"/>
       <c r="D253" s="7"/>
       <c r="E253" s="7">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="F253" s="294"/>
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="F253" s="293">
+        <f>SUM(E253:E263)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="254" s="249" customFormat="1" spans="1:6">
-      <c r="A254" s="287"/>
+      <c r="A254" s="286"/>
       <c r="B254" s="290"/>
       <c r="C254" s="297"/>
       <c r="D254" s="7"/>
       <c r="E254" s="7">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="F254" s="295"/>
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="F254" s="294"/>
     </row>
     <row r="255" s="249" customFormat="1" spans="1:6">
-      <c r="A255" s="283"/>
+      <c r="A255" s="286"/>
       <c r="B255" s="290"/>
       <c r="C255" s="297"/>
       <c r="D255" s="7"/>
       <c r="E255" s="7">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="F255" s="293">
-        <f>SUM(E255:E265)</f>
-        <v>0</v>
-      </c>
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="F255" s="294"/>
     </row>
     <row r="256" s="249" customFormat="1" spans="1:6">
       <c r="A256" s="286"/>
@@ -7011,7 +7174,7 @@
       <c r="C256" s="297"/>
       <c r="D256" s="7"/>
       <c r="E256" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="F256" s="294"/>
@@ -7022,7 +7185,7 @@
       <c r="C257" s="297"/>
       <c r="D257" s="7"/>
       <c r="E257" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="F257" s="294"/>
@@ -7033,7 +7196,7 @@
       <c r="C258" s="297"/>
       <c r="D258" s="7"/>
       <c r="E258" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="F258" s="294"/>
@@ -7044,7 +7207,7 @@
       <c r="C259" s="297"/>
       <c r="D259" s="7"/>
       <c r="E259" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="F259" s="294"/>
@@ -7055,7 +7218,7 @@
       <c r="C260" s="297"/>
       <c r="D260" s="7"/>
       <c r="E260" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="F260" s="294"/>
@@ -7066,7 +7229,7 @@
       <c r="C261" s="297"/>
       <c r="D261" s="7"/>
       <c r="E261" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="F261" s="294"/>
@@ -7077,57 +7240,57 @@
       <c r="C262" s="297"/>
       <c r="D262" s="7"/>
       <c r="E262" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="F262" s="294"/>
     </row>
     <row r="263" s="249" customFormat="1" spans="1:6">
-      <c r="A263" s="286"/>
+      <c r="A263" s="287"/>
       <c r="B263" s="290"/>
       <c r="C263" s="297"/>
       <c r="D263" s="7"/>
       <c r="E263" s="7">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="F263" s="294"/>
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="F263" s="295"/>
     </row>
     <row r="264" s="249" customFormat="1" spans="1:6">
-      <c r="A264" s="286"/>
+      <c r="A264" s="283"/>
       <c r="B264" s="290"/>
       <c r="C264" s="297"/>
       <c r="D264" s="7"/>
       <c r="E264" s="7">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="F264" s="294"/>
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="F264" s="293">
+        <f>SUM(E264:E274)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="265" s="249" customFormat="1" spans="1:6">
-      <c r="A265" s="287"/>
+      <c r="A265" s="286"/>
       <c r="B265" s="290"/>
       <c r="C265" s="297"/>
       <c r="D265" s="7"/>
       <c r="E265" s="7">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="F265" s="295"/>
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="F265" s="294"/>
     </row>
     <row r="266" s="249" customFormat="1" spans="1:6">
-      <c r="A266" s="283"/>
+      <c r="A266" s="286"/>
       <c r="B266" s="290"/>
       <c r="C266" s="297"/>
       <c r="D266" s="7"/>
       <c r="E266" s="7">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="F266" s="293">
-        <f>SUM(E266:E275)</f>
-        <v>0</v>
-      </c>
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="F266" s="294"/>
     </row>
     <row r="267" s="249" customFormat="1" spans="1:6">
       <c r="A267" s="286"/>
@@ -7135,7 +7298,7 @@
       <c r="C267" s="297"/>
       <c r="D267" s="7"/>
       <c r="E267" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="F267" s="294"/>
@@ -7146,7 +7309,7 @@
       <c r="C268" s="297"/>
       <c r="D268" s="7"/>
       <c r="E268" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="F268" s="294"/>
@@ -7157,7 +7320,7 @@
       <c r="C269" s="297"/>
       <c r="D269" s="7"/>
       <c r="E269" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="F269" s="294"/>
@@ -7168,7 +7331,7 @@
       <c r="C270" s="297"/>
       <c r="D270" s="7"/>
       <c r="E270" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="F270" s="294"/>
@@ -7179,7 +7342,7 @@
       <c r="C271" s="297"/>
       <c r="D271" s="7"/>
       <c r="E271" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="F271" s="294"/>
@@ -7190,7 +7353,7 @@
       <c r="C272" s="297"/>
       <c r="D272" s="7"/>
       <c r="E272" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="F272" s="294"/>
@@ -7201,24 +7364,24 @@
       <c r="C273" s="297"/>
       <c r="D273" s="7"/>
       <c r="E273" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="F273" s="294"/>
     </row>
     <row r="274" s="249" customFormat="1" spans="1:6">
-      <c r="A274" s="286"/>
+      <c r="A274" s="287"/>
       <c r="B274" s="290"/>
       <c r="C274" s="297"/>
       <c r="D274" s="7"/>
       <c r="E274" s="7">
-        <f t="shared" ref="E274:E287" si="8">SUM(C274*D274)</f>
-        <v>0</v>
-      </c>
-      <c r="F274" s="294"/>
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="F274" s="295"/>
     </row>
     <row r="275" s="249" customFormat="1" spans="1:6">
-      <c r="A275" s="287"/>
+      <c r="A275" s="283"/>
       <c r="B275" s="290"/>
       <c r="C275" s="297"/>
       <c r="D275" s="7"/>
@@ -7226,10 +7389,13 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="F275" s="295"/>
-    </row>
-    <row r="276" s="249" customFormat="1" ht="17.6" spans="1:6">
-      <c r="A276" s="291"/>
+      <c r="F275" s="293">
+        <f>SUM(E275:E284)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="276" s="249" customFormat="1" spans="1:6">
+      <c r="A276" s="286"/>
       <c r="B276" s="290"/>
       <c r="C276" s="297"/>
       <c r="D276" s="7"/>
@@ -7237,13 +7403,10 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="F276" s="298">
-        <f>SUM(E276)</f>
-        <v>0</v>
-      </c>
+      <c r="F276" s="294"/>
     </row>
     <row r="277" s="249" customFormat="1" spans="1:6">
-      <c r="A277" s="283"/>
+      <c r="A277" s="286"/>
       <c r="B277" s="290"/>
       <c r="C277" s="297"/>
       <c r="D277" s="7"/>
@@ -7251,10 +7414,7 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="F277" s="293">
-        <f>SUM(E277:E287)</f>
-        <v>0</v>
-      </c>
+      <c r="F277" s="294"/>
     </row>
     <row r="278" s="249" customFormat="1" spans="1:6">
       <c r="A278" s="286"/>
@@ -7317,99 +7477,168 @@
       <c r="C283" s="297"/>
       <c r="D283" s="7"/>
       <c r="E283" s="7">
-        <f t="shared" si="8"/>
+        <f t="shared" ref="E283:E296" si="9">SUM(C283*D283)</f>
         <v>0</v>
       </c>
       <c r="F283" s="294"/>
     </row>
     <row r="284" s="249" customFormat="1" spans="1:6">
-      <c r="A284" s="286"/>
+      <c r="A284" s="287"/>
       <c r="B284" s="290"/>
       <c r="C284" s="297"/>
       <c r="D284" s="7"/>
       <c r="E284" s="7">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="F284" s="294"/>
-    </row>
-    <row r="285" s="249" customFormat="1" spans="1:6">
-      <c r="A285" s="286"/>
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="F284" s="295"/>
+    </row>
+    <row r="285" s="249" customFormat="1" ht="17.6" spans="1:6">
+      <c r="A285" s="291"/>
       <c r="B285" s="290"/>
       <c r="C285" s="297"/>
       <c r="D285" s="7"/>
       <c r="E285" s="7">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="F285" s="294"/>
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="F285" s="306">
+        <f>SUM(E285)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="286" s="249" customFormat="1" spans="1:6">
-      <c r="A286" s="286"/>
+      <c r="A286" s="283"/>
       <c r="B286" s="290"/>
       <c r="C286" s="297"/>
       <c r="D286" s="7"/>
       <c r="E286" s="7">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="F286" s="294"/>
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="F286" s="293">
+        <f>SUM(E286:E296)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="287" s="249" customFormat="1" spans="1:6">
-      <c r="A287" s="287"/>
+      <c r="A287" s="286"/>
       <c r="B287" s="290"/>
       <c r="C287" s="297"/>
       <c r="D287" s="7"/>
       <c r="E287" s="7">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="F287" s="295"/>
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="F287" s="294"/>
     </row>
     <row r="288" s="249" customFormat="1" spans="1:6">
-      <c r="A288" s="251"/>
-      <c r="C288" s="250"/>
-      <c r="E288" s="7"/>
-      <c r="F288" s="298">
-        <f>SUM(F2:F287)</f>
-        <v>3916000</v>
-      </c>
-    </row>
-    <row r="289" s="249" customFormat="1" spans="1:3">
-      <c r="A289" s="251"/>
-      <c r="C289" s="250"/>
-    </row>
-    <row r="290" s="249" customFormat="1" spans="1:3">
-      <c r="A290" s="251"/>
-      <c r="C290" s="250"/>
-    </row>
-    <row r="291" s="249" customFormat="1" spans="1:3">
-      <c r="A291" s="251"/>
-      <c r="C291" s="250"/>
-    </row>
-    <row r="292" s="249" customFormat="1" spans="1:3">
-      <c r="A292" s="251"/>
-      <c r="C292" s="250"/>
-    </row>
-    <row r="293" s="249" customFormat="1" spans="1:3">
-      <c r="A293" s="251"/>
-      <c r="C293" s="250"/>
-    </row>
-    <row r="294" s="249" customFormat="1" spans="1:3">
-      <c r="A294" s="251"/>
-      <c r="C294" s="250"/>
-    </row>
-    <row r="295" s="249" customFormat="1" spans="1:3">
-      <c r="A295" s="251"/>
-      <c r="C295" s="250"/>
-    </row>
-    <row r="296" s="249" customFormat="1" spans="1:3">
-      <c r="A296" s="251"/>
-      <c r="C296" s="250"/>
-    </row>
-    <row r="297" s="249" customFormat="1" spans="1:3">
+      <c r="A288" s="286"/>
+      <c r="B288" s="290"/>
+      <c r="C288" s="297"/>
+      <c r="D288" s="7"/>
+      <c r="E288" s="7">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="F288" s="294"/>
+    </row>
+    <row r="289" s="249" customFormat="1" spans="1:6">
+      <c r="A289" s="286"/>
+      <c r="B289" s="290"/>
+      <c r="C289" s="297"/>
+      <c r="D289" s="7"/>
+      <c r="E289" s="7">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="F289" s="294"/>
+    </row>
+    <row r="290" s="249" customFormat="1" spans="1:6">
+      <c r="A290" s="286"/>
+      <c r="B290" s="290"/>
+      <c r="C290" s="297"/>
+      <c r="D290" s="7"/>
+      <c r="E290" s="7">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="F290" s="294"/>
+    </row>
+    <row r="291" s="249" customFormat="1" spans="1:6">
+      <c r="A291" s="286"/>
+      <c r="B291" s="290"/>
+      <c r="C291" s="297"/>
+      <c r="D291" s="7"/>
+      <c r="E291" s="7">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="F291" s="294"/>
+    </row>
+    <row r="292" s="249" customFormat="1" spans="1:6">
+      <c r="A292" s="286"/>
+      <c r="B292" s="290"/>
+      <c r="C292" s="297"/>
+      <c r="D292" s="7"/>
+      <c r="E292" s="7">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="F292" s="294"/>
+    </row>
+    <row r="293" s="249" customFormat="1" spans="1:6">
+      <c r="A293" s="286"/>
+      <c r="B293" s="290"/>
+      <c r="C293" s="297"/>
+      <c r="D293" s="7"/>
+      <c r="E293" s="7">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="F293" s="294"/>
+    </row>
+    <row r="294" s="249" customFormat="1" spans="1:6">
+      <c r="A294" s="286"/>
+      <c r="B294" s="290"/>
+      <c r="C294" s="297"/>
+      <c r="D294" s="7"/>
+      <c r="E294" s="7">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="F294" s="294"/>
+    </row>
+    <row r="295" s="249" customFormat="1" spans="1:6">
+      <c r="A295" s="286"/>
+      <c r="B295" s="290"/>
+      <c r="C295" s="297"/>
+      <c r="D295" s="7"/>
+      <c r="E295" s="7">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="F295" s="294"/>
+    </row>
+    <row r="296" s="249" customFormat="1" spans="1:6">
+      <c r="A296" s="287"/>
+      <c r="B296" s="290"/>
+      <c r="C296" s="297"/>
+      <c r="D296" s="7"/>
+      <c r="E296" s="7">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="F296" s="295"/>
+    </row>
+    <row r="297" s="249" customFormat="1" spans="1:6">
       <c r="A297" s="251"/>
       <c r="C297" s="250"/>
+      <c r="E297" s="7"/>
+      <c r="F297" s="306">
+        <f>SUM(F2:F296)</f>
+        <v>5052000</v>
+      </c>
     </row>
     <row r="298" s="249" customFormat="1" spans="1:3">
       <c r="A298" s="251"/>
@@ -7783,13 +8012,49 @@
       <c r="A390" s="251"/>
       <c r="C390" s="250"/>
     </row>
-    <row r="391" s="249" customFormat="1" spans="1:7">
+    <row r="391" s="249" customFormat="1" spans="1:3">
       <c r="A391" s="251"/>
       <c r="C391" s="250"/>
-      <c r="G391" s="275"/>
+    </row>
+    <row r="392" s="249" customFormat="1" spans="1:3">
+      <c r="A392" s="251"/>
+      <c r="C392" s="250"/>
+    </row>
+    <row r="393" s="249" customFormat="1" spans="1:3">
+      <c r="A393" s="251"/>
+      <c r="C393" s="250"/>
+    </row>
+    <row r="394" s="249" customFormat="1" spans="1:3">
+      <c r="A394" s="251"/>
+      <c r="C394" s="250"/>
+    </row>
+    <row r="395" s="249" customFormat="1" spans="1:3">
+      <c r="A395" s="251"/>
+      <c r="C395" s="250"/>
+    </row>
+    <row r="396" s="249" customFormat="1" spans="1:3">
+      <c r="A396" s="251"/>
+      <c r="C396" s="250"/>
+    </row>
+    <row r="397" s="249" customFormat="1" spans="1:3">
+      <c r="A397" s="251"/>
+      <c r="C397" s="250"/>
+    </row>
+    <row r="398" s="249" customFormat="1" spans="1:3">
+      <c r="A398" s="251"/>
+      <c r="C398" s="250"/>
+    </row>
+    <row r="399" s="249" customFormat="1" spans="1:3">
+      <c r="A399" s="251"/>
+      <c r="C399" s="250"/>
+    </row>
+    <row r="400" s="249" customFormat="1" spans="1:7">
+      <c r="A400" s="251"/>
+      <c r="C400" s="250"/>
+      <c r="G400" s="275"/>
     </row>
   </sheetData>
-  <mergeCells count="36">
+  <mergeCells count="40">
     <mergeCell ref="A2:A12"/>
     <mergeCell ref="A13:A25"/>
     <mergeCell ref="A26:A34"/>
@@ -7800,14 +8065,16 @@
     <mergeCell ref="A68:A78"/>
     <mergeCell ref="A79:A93"/>
     <mergeCell ref="A94:A99"/>
-    <mergeCell ref="A204:A211"/>
-    <mergeCell ref="A212:A223"/>
-    <mergeCell ref="A224:A232"/>
-    <mergeCell ref="A233:A243"/>
-    <mergeCell ref="A244:A254"/>
-    <mergeCell ref="A255:A265"/>
-    <mergeCell ref="A266:A275"/>
-    <mergeCell ref="A277:A287"/>
+    <mergeCell ref="A100:A108"/>
+    <mergeCell ref="A109:A121"/>
+    <mergeCell ref="A213:A220"/>
+    <mergeCell ref="A221:A232"/>
+    <mergeCell ref="A233:A241"/>
+    <mergeCell ref="A242:A252"/>
+    <mergeCell ref="A253:A263"/>
+    <mergeCell ref="A264:A274"/>
+    <mergeCell ref="A275:A284"/>
+    <mergeCell ref="A286:A296"/>
     <mergeCell ref="F2:F12"/>
     <mergeCell ref="F13:F25"/>
     <mergeCell ref="F26:F34"/>
@@ -7818,14 +8085,16 @@
     <mergeCell ref="F68:F78"/>
     <mergeCell ref="F79:F93"/>
     <mergeCell ref="F94:F99"/>
-    <mergeCell ref="F204:F211"/>
-    <mergeCell ref="F212:F223"/>
-    <mergeCell ref="F224:F232"/>
-    <mergeCell ref="F233:F243"/>
-    <mergeCell ref="F244:F254"/>
-    <mergeCell ref="F255:F265"/>
-    <mergeCell ref="F266:F275"/>
-    <mergeCell ref="F277:F287"/>
+    <mergeCell ref="F100:F108"/>
+    <mergeCell ref="F109:F121"/>
+    <mergeCell ref="F213:F220"/>
+    <mergeCell ref="F221:F232"/>
+    <mergeCell ref="F233:F241"/>
+    <mergeCell ref="F242:F252"/>
+    <mergeCell ref="F253:F263"/>
+    <mergeCell ref="F264:F274"/>
+    <mergeCell ref="F275:F284"/>
+    <mergeCell ref="F286:F296"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
@@ -7852,16 +8121,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="35" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C1" s="35" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="D1" s="35" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="E1" s="35" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="F1" s="35" t="s">
         <v>3</v>
@@ -7878,7 +8147,7 @@
         <v>38678</v>
       </c>
       <c r="C2" s="38" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D2" s="27">
         <v>3</v>
@@ -7901,7 +8170,7 @@
       <c r="D3" s="27"/>
       <c r="E3" s="17"/>
       <c r="F3" s="123" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="G3" s="53">
         <f>G2*11%</f>
@@ -7943,7 +8212,7 @@
       <c r="D6" s="122"/>
       <c r="E6" s="7"/>
       <c r="F6" s="127" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="G6" s="7">
         <f>G5*11%</f>
@@ -8025,7 +8294,7 @@
     </row>
     <row r="14" ht="24" customHeight="1" spans="1:7">
       <c r="A14" s="81" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="B14" s="82"/>
       <c r="C14" s="82"/>
@@ -8080,16 +8349,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="35" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C1" s="35" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="D1" s="35" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="E1" s="35" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="F1" s="35" t="s">
         <v>3</v>
@@ -8228,7 +8497,7 @@
     </row>
     <row r="14" ht="24" customHeight="1" spans="1:7">
       <c r="A14" s="81" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="B14" s="82"/>
       <c r="C14" s="82"/>
@@ -8282,16 +8551,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="35" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C1" s="35" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="D1" s="35" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="E1" s="35" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="F1" s="35" t="s">
         <v>3</v>
@@ -8300,7 +8569,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="35" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="2" ht="147.55" customHeight="1" spans="1:8">
@@ -8308,10 +8577,10 @@
         <v>45999</v>
       </c>
       <c r="B2" s="93" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C2" s="69" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D2" s="56">
         <v>24</v>
@@ -8338,7 +8607,7 @@
       </c>
       <c r="E3" s="106"/>
       <c r="F3" s="86" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="G3" s="107">
         <f>G2*11%</f>
@@ -8386,7 +8655,7 @@
       </c>
       <c r="E6" s="85"/>
       <c r="F6" s="86" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="G6" s="107">
         <f>G5*11%</f>
@@ -8431,7 +8700,7 @@
       <c r="D9" s="102"/>
       <c r="E9" s="85"/>
       <c r="F9" s="86" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="G9" s="107">
         <f>G8*11%</f>
@@ -8476,7 +8745,7 @@
       <c r="D12" s="102"/>
       <c r="E12" s="85"/>
       <c r="F12" s="86" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="G12" s="107">
         <f>G11*11%</f>
@@ -8518,7 +8787,7 @@
       <c r="D15" s="102"/>
       <c r="E15" s="85"/>
       <c r="F15" s="86" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="G15" s="107">
         <f>G14*11%</f>
@@ -8543,7 +8812,7 @@
     </row>
     <row r="17" ht="26" customHeight="1" spans="1:8">
       <c r="A17" s="81" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="B17" s="82"/>
       <c r="C17" s="82"/>
@@ -8602,19 +8871,19 @@
         <v>0</v>
       </c>
       <c r="B1" s="35" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C1" s="35" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="D1" s="35" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E1" s="35" t="s">
         <v>3</v>
       </c>
       <c r="F1" s="35" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="G1" s="35" t="s">
         <v>5</v>
@@ -8646,7 +8915,7 @@
     </row>
     <row r="4" ht="23" customHeight="1" spans="1:7">
       <c r="A4" s="94" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B4" s="95"/>
       <c r="C4" s="95"/>
@@ -8687,16 +8956,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="35" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C1" s="35" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="D1" s="35" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E1" s="35" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="F1" s="35" t="s">
         <v>3</v>
@@ -8710,10 +8979,10 @@
         <v>45999</v>
       </c>
       <c r="B2" s="77" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C2" s="26" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D2" s="27">
         <v>3</v>
@@ -8729,7 +8998,7 @@
     </row>
     <row r="3" ht="26" spans="1:7">
       <c r="A3" s="28" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B3" s="29"/>
       <c r="C3" s="78"/>
@@ -8739,7 +9008,7 @@
       </c>
       <c r="E3" s="85"/>
       <c r="F3" s="85" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="G3" s="86">
         <f>G2*11%</f>
@@ -8794,7 +9063,7 @@
     </row>
     <row r="8" ht="26" customHeight="1" spans="1:7">
       <c r="A8" s="81" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="B8" s="82"/>
       <c r="C8" s="82"/>
@@ -8842,19 +9111,19 @@
         <v>0</v>
       </c>
       <c r="B1" s="13" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C1" s="13" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="D1" s="13" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="E1" s="13" t="s">
         <v>5</v>
       </c>
       <c r="F1" s="13" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="2" ht="321" customHeight="1" spans="1:6">
@@ -8917,16 +9186,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="35" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C1" s="35" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="D1" s="35" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E1" s="35" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="F1" s="35" t="s">
         <v>3</v>
@@ -9027,7 +9296,7 @@
     </row>
     <row r="12" ht="27" customHeight="1" spans="1:7">
       <c r="A12" s="49" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="B12" s="50"/>
       <c r="C12" s="50"/>
@@ -9080,13 +9349,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="13" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C1" s="13" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D1" s="13" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="E1" s="13" t="s">
         <v>3</v>
@@ -9095,7 +9364,7 @@
         <v>5</v>
       </c>
       <c r="G1" s="13" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="2" ht="324.4" customHeight="1" spans="1:7">
@@ -9154,22 +9423,22 @@
         <v>0</v>
       </c>
       <c r="B1" s="13" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C1" s="13" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D1" s="13" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="E1" s="13" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="F1" s="13" t="s">
         <v>5</v>
       </c>
       <c r="G1" s="13" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="2" ht="177" customHeight="1" spans="1:7">
@@ -9230,10 +9499,10 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C1" s="3" t="s">
         <v>5</v>
@@ -9244,11 +9513,11 @@
         <v>1</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C2" s="5">
-        <f>'BUK BUNGA (Groceries)'!F288</f>
-        <v>3916000</v>
+        <f>'BUK BUNGA (Groceries)'!F297</f>
+        <v>5052000</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -9256,7 +9525,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="C3" s="5">
         <f>'WARUNG EKA (Drinks, Etc)'!G117</f>
@@ -9268,7 +9537,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C4" s="5">
         <f>'DEWATA COCONUT (Coconut)'!E10</f>
@@ -9280,7 +9549,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C5" s="5">
         <f>'SEDANA JAYA'!F37</f>
@@ -9292,7 +9561,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C6" s="5">
         <f>'PNB (Alcohol)'!H7</f>
@@ -9304,7 +9573,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C7" s="5">
         <f>'DSP (Alcohol)'!F16</f>
@@ -9316,7 +9585,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C8" s="5">
         <f>'DSP ARYA BIMA (Alcohol)'!E3</f>
@@ -9328,7 +9597,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C9" s="5" t="str">
         <f>'SELERA OR STIR UP (Syrup)'!F19</f>
@@ -9340,7 +9609,7 @@
         <v>9</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="C10" s="5">
         <f>'DW BALI (Alcohol)'!E6</f>
@@ -9352,7 +9621,7 @@
         <v>10</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C11" s="5">
         <f>'DDB (Alcohol)'!E14</f>
@@ -9364,7 +9633,7 @@
         <v>11</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C12" s="5">
         <f>'NANO DEWATA (Alcohol)'!E14</f>
@@ -9376,7 +9645,7 @@
         <v>12</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="C13" s="5">
         <f>'BALI PERMATA JAYA (Corona Beer)'!E17</f>
@@ -9388,7 +9657,7 @@
         <v>13</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C14" s="7">
         <f>'BLACK COFFEE ROASTERS (Coffee)'!F4</f>
@@ -9400,7 +9669,7 @@
         <v>14</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="C15" s="5">
         <f>'PT. PRASIDA LANTUR MAJU (Wine)'!E8</f>
@@ -9412,7 +9681,7 @@
         <v>15</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C16" s="8">
         <f>'PT LOVINA BEACH BREWERY'!D3</f>
@@ -9424,7 +9693,7 @@
         <v>16</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C17" s="5">
         <f>'CHAI CHITAI (Tea Leaf,etc)'!E12</f>
@@ -9436,7 +9705,7 @@
         <v>17</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="C18" s="5">
         <f>'MULIA JAYA (Passion Fruit)'!D3</f>
@@ -9448,7 +9717,7 @@
         <v>18</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C19" s="5">
         <f>'Dewata Kencana Distribusi (Vdka'!E3</f>
@@ -9462,7 +9731,7 @@
       <c r="B20" s="9"/>
       <c r="C20" s="10">
         <f>SUM(C2:C13)</f>
-        <v>17668109.94</v>
+        <v>18804109.94</v>
       </c>
     </row>
   </sheetData>
@@ -9498,7 +9767,7 @@
   <sheetData>
     <row r="1" s="249" customFormat="1" ht="21" customHeight="1" spans="1:7">
       <c r="A1" s="255" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="B1" s="256" t="s">
         <v>0</v>
@@ -9513,10 +9782,10 @@
         <v>3</v>
       </c>
       <c r="F1" s="257" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="G1" s="257" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
     </row>
     <row r="2" s="249" customFormat="1" ht="19" customHeight="1" spans="1:7">
@@ -9527,7 +9796,7 @@
         <v>45992</v>
       </c>
       <c r="C2" s="259" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="D2" s="115">
         <v>5</v>
@@ -9548,7 +9817,7 @@
       <c r="A3" s="41"/>
       <c r="B3" s="40"/>
       <c r="C3" s="259" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="D3" s="115">
         <v>1</v>
@@ -9566,7 +9835,7 @@
       <c r="A4" s="260"/>
       <c r="B4" s="131"/>
       <c r="C4" s="259" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="D4" s="115">
         <v>1</v>
@@ -9588,7 +9857,7 @@
         <v>45993</v>
       </c>
       <c r="C5" s="259" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="D5" s="115">
         <v>5</v>
@@ -9609,7 +9878,7 @@
       <c r="A6" s="209"/>
       <c r="B6" s="40"/>
       <c r="C6" s="259" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="D6" s="115">
         <v>1</v>
@@ -9627,7 +9896,7 @@
       <c r="A7" s="207"/>
       <c r="B7" s="131"/>
       <c r="C7" s="259" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="D7" s="115">
         <v>1</v>
@@ -9649,7 +9918,7 @@
         <v>45994</v>
       </c>
       <c r="C8" s="259" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="D8" s="115">
         <v>6</v>
@@ -9670,7 +9939,7 @@
       <c r="A9" s="209"/>
       <c r="B9" s="40"/>
       <c r="C9" s="259" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="D9" s="115">
         <v>1</v>
@@ -9688,7 +9957,7 @@
       <c r="A10" s="209"/>
       <c r="B10" s="40"/>
       <c r="C10" s="259" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="D10" s="115">
         <v>1</v>
@@ -9706,7 +9975,7 @@
       <c r="A11" s="209"/>
       <c r="B11" s="40"/>
       <c r="C11" s="259" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="D11" s="115">
         <v>1</v>
@@ -9724,7 +9993,7 @@
       <c r="A12" s="209"/>
       <c r="B12" s="40"/>
       <c r="C12" s="261" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="D12" s="115">
         <v>2</v>
@@ -9742,7 +10011,7 @@
       <c r="A13" s="207"/>
       <c r="B13" s="131"/>
       <c r="C13" s="259" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D13" s="115">
         <v>1</v>
@@ -9764,7 +10033,7 @@
         <v>45995</v>
       </c>
       <c r="C14" s="259" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="D14" s="115">
         <v>6</v>
@@ -9785,7 +10054,7 @@
       <c r="A15" s="207"/>
       <c r="B15" s="131"/>
       <c r="C15" s="261" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="D15" s="115">
         <v>2</v>
@@ -9807,7 +10076,7 @@
         <v>45997</v>
       </c>
       <c r="C16" s="261" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="D16" s="115">
         <v>2</v>
@@ -9828,7 +10097,7 @@
       <c r="A17" s="209"/>
       <c r="B17" s="40"/>
       <c r="C17" s="261" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="D17" s="115">
         <v>1</v>
@@ -9846,7 +10115,7 @@
       <c r="A18" s="207"/>
       <c r="B18" s="131"/>
       <c r="C18" s="261" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="D18" s="115">
         <v>5</v>
@@ -9868,7 +10137,7 @@
         <v>45998</v>
       </c>
       <c r="C19" s="259" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="D19" s="115">
         <v>2</v>
@@ -9889,7 +10158,7 @@
       <c r="A20" s="209"/>
       <c r="B20" s="40"/>
       <c r="C20" s="259" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="D20" s="115">
         <v>1</v>
@@ -9907,7 +10176,7 @@
       <c r="A21" s="209"/>
       <c r="B21" s="40"/>
       <c r="C21" s="259" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="D21" s="115">
         <v>5</v>
@@ -9925,7 +10194,7 @@
       <c r="A22" s="209"/>
       <c r="B22" s="40"/>
       <c r="C22" s="259" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="D22" s="115">
         <v>1</v>
@@ -9943,7 +10212,7 @@
       <c r="A23" s="207"/>
       <c r="B23" s="131"/>
       <c r="C23" s="261" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="D23" s="115">
         <v>2</v>
@@ -9965,7 +10234,7 @@
         <v>45999</v>
       </c>
       <c r="C24" s="259" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="D24" s="115">
         <v>1</v>
@@ -9986,7 +10255,7 @@
       <c r="A25" s="209"/>
       <c r="B25" s="40"/>
       <c r="C25" s="259" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D25" s="115">
         <v>1</v>
@@ -10004,7 +10273,7 @@
       <c r="A26" s="209"/>
       <c r="B26" s="40"/>
       <c r="C26" s="261" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="D26" s="115">
         <v>1</v>
@@ -10022,7 +10291,7 @@
       <c r="A27" s="207"/>
       <c r="B27" s="131"/>
       <c r="C27" s="259" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="D27" s="115">
         <v>4</v>
@@ -10044,7 +10313,7 @@
         <v>46000</v>
       </c>
       <c r="C28" s="261" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="D28" s="115">
         <v>5</v>
@@ -10065,7 +10334,7 @@
       <c r="A29" s="209"/>
       <c r="B29" s="40"/>
       <c r="C29" s="259" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="D29" s="115">
         <v>1</v>
@@ -10083,7 +10352,7 @@
       <c r="A30" s="207"/>
       <c r="B30" s="131"/>
       <c r="C30" s="259" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="D30" s="115">
         <v>1</v>
@@ -10105,7 +10374,7 @@
         <v>46001</v>
       </c>
       <c r="C31" s="262" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="D31" s="115">
         <v>6</v>
@@ -10126,7 +10395,7 @@
       <c r="A32" s="56"/>
       <c r="B32" s="25"/>
       <c r="C32" s="263" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="D32" s="115">
         <v>1</v>
@@ -10144,7 +10413,7 @@
       <c r="A33" s="56"/>
       <c r="B33" s="25"/>
       <c r="C33" s="262" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="D33" s="115">
         <v>1</v>
@@ -10162,7 +10431,7 @@
       <c r="A34" s="56"/>
       <c r="B34" s="25"/>
       <c r="C34" s="262" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="D34" s="115">
         <v>1</v>
@@ -10180,7 +10449,7 @@
       <c r="A35" s="56"/>
       <c r="B35" s="25"/>
       <c r="C35" s="262" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D35" s="115">
         <v>1</v>
@@ -10198,7 +10467,7 @@
       <c r="A36" s="56"/>
       <c r="B36" s="25"/>
       <c r="C36" s="262" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="D36" s="115">
         <v>1</v>
@@ -10216,7 +10485,7 @@
       <c r="A37" s="56"/>
       <c r="B37" s="25"/>
       <c r="C37" s="262" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="D37" s="115">
         <v>2</v>
@@ -10238,7 +10507,7 @@
         <v>46002</v>
       </c>
       <c r="C38" s="259" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="D38" s="115">
         <v>6</v>
@@ -10259,7 +10528,7 @@
       <c r="A39" s="209"/>
       <c r="B39" s="40"/>
       <c r="C39" s="259" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="D39" s="115">
         <v>2</v>
@@ -10277,7 +10546,7 @@
       <c r="A40" s="209"/>
       <c r="B40" s="40"/>
       <c r="C40" s="259" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="D40" s="115">
         <v>1</v>
@@ -10299,7 +10568,7 @@
         <v>46003</v>
       </c>
       <c r="C41" s="259" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="D41" s="115">
         <v>6</v>
@@ -10320,7 +10589,7 @@
       <c r="A42" s="209"/>
       <c r="B42" s="40"/>
       <c r="C42" s="259" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="D42" s="115">
         <v>1</v>
@@ -10338,7 +10607,7 @@
       <c r="A43" s="209"/>
       <c r="B43" s="40"/>
       <c r="C43" s="259" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="D43" s="115">
         <v>2</v>
@@ -10356,7 +10625,7 @@
       <c r="A44" s="209"/>
       <c r="B44" s="40"/>
       <c r="C44" s="259" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="D44" s="115">
         <v>1</v>
@@ -10374,7 +10643,7 @@
       <c r="A45" s="207"/>
       <c r="B45" s="131"/>
       <c r="C45" s="259" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D45" s="115">
         <v>1</v>
@@ -10396,7 +10665,7 @@
         <v>46004</v>
       </c>
       <c r="C46" s="259" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="D46" s="115">
         <v>1</v>
@@ -10417,7 +10686,7 @@
       <c r="A47" s="207"/>
       <c r="B47" s="131"/>
       <c r="C47" s="259" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="D47" s="115">
         <v>6</v>
@@ -11332,7 +11601,7 @@
     </row>
     <row r="117" s="249" customFormat="1" spans="1:7">
       <c r="A117" s="273" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="B117" s="122"/>
       <c r="C117" s="274"/>
@@ -11717,16 +11986,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="13" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C1" s="13" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="D1" s="13" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="E1" s="13" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="F1" s="13" t="s">
         <v>3</v>
@@ -11743,7 +12012,7 @@
         <v>12340</v>
       </c>
       <c r="C2" s="69" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="D2" s="16">
         <v>20</v>
@@ -11765,7 +12034,7 @@
         <v>12357</v>
       </c>
       <c r="C3" s="69" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="D3" s="16">
         <v>20</v>
@@ -11787,7 +12056,7 @@
         <v>11374</v>
       </c>
       <c r="C4" s="69" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="D4" s="16">
         <v>20</v>
@@ -11809,7 +12078,7 @@
         <v>13396</v>
       </c>
       <c r="C5" s="69" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="D5" s="16">
         <v>20</v>
@@ -11831,7 +12100,7 @@
         <v>11474</v>
       </c>
       <c r="C6" s="69" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="D6" s="16">
         <v>20</v>
@@ -11939,7 +12208,7 @@
         <v>3</v>
       </c>
       <c r="E1" s="229" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="F1" s="229" t="s">
         <v>5</v>
@@ -11987,7 +12256,7 @@
     <row r="4" s="222" customFormat="1" spans="1:7">
       <c r="A4" s="234"/>
       <c r="B4" s="231" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C4" s="232">
         <v>0.3</v>
@@ -12005,7 +12274,7 @@
     <row r="5" s="222" customFormat="1" spans="1:6">
       <c r="A5" s="234"/>
       <c r="B5" s="231" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="C5" s="232">
         <v>1</v>
@@ -12091,7 +12360,7 @@
     <row r="10" s="222" customFormat="1" spans="1:6">
       <c r="A10" s="235"/>
       <c r="B10" s="231" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="C10" s="232">
         <v>2</v>
@@ -12148,7 +12417,7 @@
     <row r="13" s="222" customFormat="1" spans="1:6">
       <c r="A13" s="234"/>
       <c r="B13" s="231" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="C13" s="232">
         <v>8</v>
@@ -12199,7 +12468,7 @@
     <row r="16" s="222" customFormat="1" spans="1:6">
       <c r="A16" s="234"/>
       <c r="B16" s="231" t="s">
-        <v>61</v>
+        <v>36</v>
       </c>
       <c r="C16" s="232">
         <v>2</v>
@@ -12233,7 +12502,7 @@
     <row r="18" s="222" customFormat="1" spans="1:6">
       <c r="A18" s="234"/>
       <c r="B18" s="231" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C18" s="232">
         <v>1</v>
@@ -12267,7 +12536,7 @@
     <row r="20" s="222" customFormat="1" spans="1:6">
       <c r="A20" s="235"/>
       <c r="B20" s="231" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C20" s="232">
         <v>1</v>
@@ -14287,19 +14556,19 @@
         <v>0</v>
       </c>
       <c r="B1" s="13" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C1" s="13" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="D1" s="13" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E1" s="13" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="F1" s="13" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="G1" s="13" t="s">
         <v>4</v>
@@ -14313,10 +14582,10 @@
         <v>45992</v>
       </c>
       <c r="B2" s="216" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C2" s="15" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D2" s="16">
         <v>3</v>
@@ -14457,31 +14726,31 @@
         <v>0</v>
       </c>
       <c r="B1" s="181" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C1" s="181" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="D1" s="181" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E1" s="181" t="s">
         <v>3</v>
       </c>
       <c r="F1" s="181" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="G1" s="181" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="H1" s="181" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="I1" s="181" t="s">
         <v>5</v>
       </c>
       <c r="J1" s="181" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="2" ht="387.45" customHeight="1" spans="1:10">
@@ -14489,10 +14758,10 @@
         <v>46000</v>
       </c>
       <c r="B2" s="183" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C2" s="175" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D2" s="184">
         <v>4</v>
@@ -14523,10 +14792,10 @@
         <v>46002</v>
       </c>
       <c r="B3" s="186" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C3" s="175" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D3" s="184">
         <v>4</v>
@@ -14556,7 +14825,7 @@
       <c r="A4" s="187"/>
       <c r="B4" s="188"/>
       <c r="C4" s="189" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D4" s="190">
         <v>4</v>
@@ -14889,16 +15158,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="172" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C1" s="172" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="D1" s="172" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E1" s="172" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="F1" s="172" t="s">
         <v>3</v>
@@ -14960,22 +15229,22 @@
         <v>0</v>
       </c>
       <c r="B1" s="141" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C1" s="141" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="D1" s="141" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E1" s="141" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="F1" s="141" t="s">
         <v>3</v>
       </c>
       <c r="G1" s="141" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="H1" s="153" t="s">
         <v>5</v>
@@ -14986,10 +15255,10 @@
         <v>45992</v>
       </c>
       <c r="B2" s="142" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="C2" s="143" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D2" s="144">
         <v>5</v>
@@ -15059,7 +15328,7 @@
       </c>
       <c r="E7" s="161"/>
       <c r="F7" s="162" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="G7" s="162"/>
       <c r="H7" s="162">
@@ -15087,10 +15356,10 @@
         <v>45999</v>
       </c>
       <c r="B9" s="142" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C9" s="151" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="D9" s="150">
         <v>3</v>
@@ -15112,7 +15381,7 @@
       <c r="A10" s="145"/>
       <c r="B10" s="145"/>
       <c r="C10" s="151" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="D10" s="150">
         <v>3</v>
@@ -15131,7 +15400,7 @@
       <c r="A11" s="152"/>
       <c r="B11" s="152"/>
       <c r="C11" s="151" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="D11" s="150">
         <v>2</v>
@@ -15158,7 +15427,7 @@
       </c>
       <c r="E12" s="161"/>
       <c r="F12" s="162" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="G12" s="162"/>
       <c r="H12" s="162">
@@ -15186,10 +15455,10 @@
         <v>45992</v>
       </c>
       <c r="B14" s="142" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="C14" s="143" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D14" s="144">
         <v>5</v>
@@ -15262,7 +15531,7 @@
       </c>
       <c r="E19" s="161"/>
       <c r="F19" s="162" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="G19" s="162"/>
       <c r="H19" s="162">
@@ -15368,22 +15637,22 @@
         <v>0</v>
       </c>
       <c r="B1" s="35" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C1" s="35" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="D1" s="34" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="E1" s="35" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="F1" s="35" t="s">
         <v>3</v>
       </c>
       <c r="G1" s="35" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="H1" s="35" t="s">
         <v>5</v>
@@ -15394,10 +15663,10 @@
         <v>46001</v>
       </c>
       <c r="B2" s="115" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C2" s="38" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="D2" s="115">
         <v>2</v>
@@ -15420,10 +15689,10 @@
         <v>46001</v>
       </c>
       <c r="B3" s="93" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C3" s="38" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D3" s="115">
         <v>4</v>
@@ -15446,10 +15715,10 @@
         <v>46004</v>
       </c>
       <c r="B4" s="130" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C4" s="38" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D4" s="115">
         <v>1</v>
@@ -15474,7 +15743,7 @@
       <c r="A5" s="131"/>
       <c r="B5" s="132"/>
       <c r="C5" s="38" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D5" s="115">
         <v>1</v>
@@ -15491,7 +15760,7 @@
     </row>
     <row r="6" ht="26" spans="1:8">
       <c r="A6" s="81" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="B6" s="82"/>
       <c r="C6" s="82"/>

</xml_diff>